<commit_message>
Implement scrollable landscape estimate workbook
</commit_message>
<xml_diff>
--- a/templates/test_cyca_estimate_single_sheet_template.xlsx
+++ b/templates/test_cyca_estimate_single_sheet_template.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="見積書" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'見積書'!$A$1:$H$182</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'見積書'!$A$1:$H$253</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;¥&quot;#,##0"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,7 +33,7 @@
       <name val="游ゴシック"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="22"/>
+      <sz val="24"/>
     </font>
     <font>
       <name val="游ゴシック"/>
@@ -57,13 +57,13 @@
       <name val="游ゴシック"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="13"/>
+      <sz val="14"/>
     </font>
     <font>
       <name val="游ゴシック"/>
       <b val="1"/>
       <color rgb="001F3557"/>
-      <sz val="20"/>
+      <sz val="22"/>
     </font>
     <font>
       <name val="游ゴシック"/>
@@ -74,11 +74,28 @@
       <name val="游ゴシック"/>
       <b val="1"/>
       <color rgb="001F3557"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="游ゴシック"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="游ゴシック"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="12"/>
     </font>
     <font>
       <name val="游ゴシック"/>
-      <sz val="9"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="游ゴシック"/>
+      <color rgb="001F3557"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="游ゴシック"/>
@@ -89,8 +106,13 @@
     <font>
       <name val="游ゴシック"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="12"/>
+      <color rgb="001F3557"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="游ゴシック"/>
+      <b val="1"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="4">
@@ -111,7 +133,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -172,12 +194,11 @@
       </bottom>
     </border>
     <border>
-      <left style="thin">
+      <top style="thin">
         <color rgb="008A97AB"/>
-      </left>
-      <right style="thin">
-        <color rgb="008A97AB"/>
-      </right>
+      </top>
+    </border>
+    <border>
       <top style="thin">
         <color rgb="008A97AB"/>
       </top>
@@ -189,7 +210,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -198,22 +219,22 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1" indent="1"/>
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -225,15 +246,15 @@
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -243,34 +264,35 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="10" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="10" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="13" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="16" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -354,7 +376,7 @@
     <from>
       <col>5</col>
       <colOff>0</colOff>
-      <row>3</row>
+      <row>2</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="1771650" cy="638175"/>
@@ -665,47 +687,46 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:H182"/>
+  <dimension ref="A2:H253"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4.5" customWidth="1" min="1" max="1"/>
-    <col width="31" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="6.5" customWidth="1" min="4" max="4"/>
-    <col width="5" customWidth="1" min="5" max="5"/>
-    <col width="11.5" customWidth="1" min="6" max="6"/>
-    <col width="14.5" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="6" customHeight="1"/>
-    <row r="2" ht="32" customHeight="1">
+    <row r="1" ht="10" customHeight="1"/>
+    <row r="2" ht="34" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
         <is>
           <t>御　見　積　書</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="4" customHeight="1"/>
-    <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="2" t="n"/>
-      <c r="D4" s="3" t="inlineStr">
+    <row r="3" ht="8" customHeight="1"/>
+    <row r="4" ht="18" customHeight="1"/>
+    <row r="5" ht="25" customHeight="1">
+      <c r="A5" s="2" t="n"/>
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>御中</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="8" customHeight="1"/>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>下記の通り御見積申し上げます。</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
+    <row r="6" ht="18" customHeight="1"/>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>下記の通りお見積もり申し上げます。</t>
+        </is>
+      </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
           <t>見積日</t>
@@ -713,7 +734,7 @@
       </c>
       <c r="G7" s="6" t="n"/>
     </row>
-    <row r="8">
+    <row r="8" ht="16" customHeight="1">
       <c r="F8" s="5" t="inlineStr">
         <is>
           <t>登録番号</t>
@@ -725,290 +746,163 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="8" customHeight="1"/>
-    <row r="10" ht="17" customHeight="1">
-      <c r="A10" s="7" t="inlineStr">
+    <row r="9" ht="18" customHeight="1"/>
+    <row r="10" ht="18" customHeight="1"/>
+    <row r="11" ht="18" customHeight="1"/>
+    <row r="12" ht="16" customHeight="1"/>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>御 見 積 金 額</t>
         </is>
       </c>
-      <c r="C10" s="8" t="n"/>
-    </row>
-    <row r="11" ht="17" customHeight="1"/>
-    <row r="12" ht="12" customHeight="1">
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C13" s="8" t="n"/>
+    </row>
+    <row r="14" ht="22" customHeight="1"/>
+    <row r="15" ht="14" customHeight="1">
+      <c r="C15" s="9" t="inlineStr">
         <is>
           <t>（消費税込）</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="10" t="inlineStr">
+    <row r="16" ht="12" customHeight="1"/>
+    <row r="17" ht="12" customHeight="1"/>
+    <row r="18" ht="12" customHeight="1"/>
+    <row r="19" ht="12" customHeight="1"/>
+    <row r="20" ht="12" customHeight="1"/>
+    <row r="21" ht="12" customHeight="1"/>
+    <row r="22" ht="12" customHeight="1"/>
+    <row r="23" ht="12" customHeight="1"/>
+    <row r="24" ht="12" customHeight="1"/>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="10" t="inlineStr">
         <is>
           <t>工事名称</t>
         </is>
       </c>
-      <c r="C13" s="11" t="n"/>
-      <c r="E13" s="12" t="inlineStr">
+      <c r="C25" s="11" t="n"/>
+      <c r="E25" s="12" t="inlineStr">
         <is>
           <t>彩架建設株式会社</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="10" t="inlineStr">
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="10" t="inlineStr">
         <is>
           <t>工事場所</t>
         </is>
       </c>
-      <c r="C14" s="11" t="n"/>
-      <c r="E14" s="13" t="inlineStr">
+      <c r="C26" s="11" t="n"/>
+      <c r="E26" s="13" t="inlineStr">
         <is>
           <t>〒839-0841 福岡県久留米市御井旗崎1丁目7-41</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="10" t="inlineStr">
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="10" t="inlineStr">
         <is>
           <t>工事期間</t>
         </is>
       </c>
-      <c r="C15" s="11" t="n"/>
-      <c r="E15" s="13" t="inlineStr">
+      <c r="C27" s="11" t="n"/>
+      <c r="E27" s="13" t="inlineStr">
         <is>
           <t>TEL 0942-65-3300　FAX 0942-65-3301</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="10" t="inlineStr">
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="10" t="inlineStr">
         <is>
           <t>支払条件</t>
         </is>
       </c>
-      <c r="C16" s="11" t="inlineStr">
+      <c r="C28" s="11" t="inlineStr">
         <is>
           <t>ご相談の上</t>
         </is>
       </c>
-      <c r="E16" s="13" t="inlineStr">
+      <c r="E28" s="13" t="inlineStr">
         <is>
           <t>代表取締役　中村 哲也</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="10" t="inlineStr">
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="10" t="inlineStr">
         <is>
           <t>有効期限</t>
         </is>
       </c>
-      <c r="C17" s="11" t="n"/>
-    </row>
-    <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="10" t="inlineStr">
+      <c r="C29" s="11" t="n"/>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="10" t="inlineStr">
         <is>
           <t>見積担当</t>
         </is>
       </c>
-      <c r="C18" s="11" t="inlineStr">
+      <c r="C30" s="11" t="inlineStr">
         <is>
           <t>中村 哲也</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="8" customHeight="1"/>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="14" t="inlineStr">
-        <is>
-          <t>工 事 内 容</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="15" t="inlineStr">
+    <row r="31" ht="12" customHeight="1"/>
+    <row r="32" ht="12" customHeight="1"/>
+    <row r="34" ht="24" customHeight="1">
+      <c r="A34" s="14" t="inlineStr">
+        <is>
+          <t>工 事 品 目 ま と め</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="15" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="B21" s="15" t="inlineStr">
+      <c r="B35" s="15" t="inlineStr">
         <is>
           <t>工事品目</t>
         </is>
       </c>
-      <c r="C21" s="15" t="inlineStr">
+      <c r="C35" s="15" t="inlineStr">
         <is>
           <t>仕様</t>
         </is>
       </c>
-      <c r="D21" s="15" t="inlineStr">
+      <c r="D35" s="15" t="inlineStr">
         <is>
           <t>数量</t>
         </is>
       </c>
-      <c r="E21" s="15" t="inlineStr">
+      <c r="E35" s="15" t="inlineStr">
         <is>
           <t>単位</t>
         </is>
       </c>
-      <c r="F21" s="15" t="inlineStr">
+      <c r="F35" s="15" t="inlineStr">
         <is>
           <t>単価</t>
         </is>
       </c>
-      <c r="G21" s="15" t="inlineStr">
+      <c r="G35" s="15" t="inlineStr">
         <is>
           <t>金額</t>
         </is>
       </c>
-      <c r="H21" s="15" t="inlineStr">
+      <c r="H35" s="15" t="inlineStr">
         <is>
           <t>備考</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="27" customHeight="1">
-      <c r="A22" s="16" t="n"/>
-      <c r="B22" s="17" t="n"/>
-      <c r="C22" s="17" t="n"/>
-      <c r="D22" s="16" t="n"/>
-      <c r="E22" s="16" t="n"/>
-      <c r="F22" s="18" t="n"/>
-      <c r="G22" s="18" t="n"/>
-      <c r="H22" s="17" t="n"/>
-    </row>
-    <row r="23" ht="27" customHeight="1">
-      <c r="A23" s="16" t="n"/>
-      <c r="B23" s="17" t="n"/>
-      <c r="C23" s="17" t="n"/>
-      <c r="D23" s="16" t="n"/>
-      <c r="E23" s="16" t="n"/>
-      <c r="F23" s="18" t="n"/>
-      <c r="G23" s="18" t="n"/>
-      <c r="H23" s="17" t="n"/>
-    </row>
-    <row r="24" ht="27" customHeight="1">
-      <c r="A24" s="16" t="n"/>
-      <c r="B24" s="17" t="n"/>
-      <c r="C24" s="17" t="n"/>
-      <c r="D24" s="16" t="n"/>
-      <c r="E24" s="16" t="n"/>
-      <c r="F24" s="18" t="n"/>
-      <c r="G24" s="18" t="n"/>
-      <c r="H24" s="17" t="n"/>
-    </row>
-    <row r="25" ht="27" customHeight="1">
-      <c r="A25" s="16" t="n"/>
-      <c r="B25" s="17" t="n"/>
-      <c r="C25" s="17" t="n"/>
-      <c r="D25" s="16" t="n"/>
-      <c r="E25" s="16" t="n"/>
-      <c r="F25" s="18" t="n"/>
-      <c r="G25" s="18" t="n"/>
-      <c r="H25" s="17" t="n"/>
-    </row>
-    <row r="26" ht="27" customHeight="1">
-      <c r="A26" s="16" t="n"/>
-      <c r="B26" s="17" t="n"/>
-      <c r="C26" s="17" t="n"/>
-      <c r="D26" s="16" t="n"/>
-      <c r="E26" s="16" t="n"/>
-      <c r="F26" s="18" t="n"/>
-      <c r="G26" s="18" t="n"/>
-      <c r="H26" s="17" t="n"/>
-    </row>
-    <row r="27" ht="27" customHeight="1">
-      <c r="A27" s="16" t="n"/>
-      <c r="B27" s="17" t="n"/>
-      <c r="C27" s="17" t="n"/>
-      <c r="D27" s="16" t="n"/>
-      <c r="E27" s="16" t="n"/>
-      <c r="F27" s="18" t="n"/>
-      <c r="G27" s="18" t="n"/>
-      <c r="H27" s="17" t="n"/>
-    </row>
-    <row r="28" ht="27" customHeight="1">
-      <c r="A28" s="16" t="n"/>
-      <c r="B28" s="17" t="n"/>
-      <c r="C28" s="17" t="n"/>
-      <c r="D28" s="16" t="n"/>
-      <c r="E28" s="16" t="n"/>
-      <c r="F28" s="18" t="n"/>
-      <c r="G28" s="18" t="n"/>
-      <c r="H28" s="17" t="n"/>
-    </row>
-    <row r="29" ht="27" customHeight="1">
-      <c r="A29" s="16" t="n"/>
-      <c r="B29" s="17" t="n"/>
-      <c r="C29" s="17" t="n"/>
-      <c r="D29" s="16" t="n"/>
-      <c r="E29" s="16" t="n"/>
-      <c r="F29" s="18" t="n"/>
-      <c r="G29" s="18" t="n"/>
-      <c r="H29" s="17" t="n"/>
-    </row>
-    <row r="30" ht="27" customHeight="1">
-      <c r="A30" s="16" t="n"/>
-      <c r="B30" s="17" t="n"/>
-      <c r="C30" s="17" t="n"/>
-      <c r="D30" s="16" t="n"/>
-      <c r="E30" s="16" t="n"/>
-      <c r="F30" s="18" t="n"/>
-      <c r="G30" s="18" t="n"/>
-      <c r="H30" s="17" t="n"/>
-    </row>
-    <row r="31" ht="27" customHeight="1">
-      <c r="A31" s="16" t="n"/>
-      <c r="B31" s="17" t="n"/>
-      <c r="C31" s="17" t="n"/>
-      <c r="D31" s="16" t="n"/>
-      <c r="E31" s="16" t="n"/>
-      <c r="F31" s="18" t="n"/>
-      <c r="G31" s="18" t="n"/>
-      <c r="H31" s="17" t="n"/>
-    </row>
-    <row r="32" ht="27" customHeight="1">
-      <c r="A32" s="16" t="n"/>
-      <c r="B32" s="17" t="n"/>
-      <c r="C32" s="17" t="n"/>
-      <c r="D32" s="16" t="n"/>
-      <c r="E32" s="16" t="n"/>
-      <c r="F32" s="18" t="n"/>
-      <c r="G32" s="18" t="n"/>
-      <c r="H32" s="17" t="n"/>
-    </row>
-    <row r="33" ht="27" customHeight="1">
-      <c r="A33" s="16" t="n"/>
-      <c r="B33" s="17" t="n"/>
-      <c r="C33" s="17" t="n"/>
-      <c r="D33" s="16" t="n"/>
-      <c r="E33" s="16" t="n"/>
-      <c r="F33" s="18" t="n"/>
-      <c r="G33" s="18" t="n"/>
-      <c r="H33" s="17" t="n"/>
-    </row>
-    <row r="34" ht="27" customHeight="1">
-      <c r="A34" s="16" t="n"/>
-      <c r="B34" s="17" t="n"/>
-      <c r="C34" s="17" t="n"/>
-      <c r="D34" s="16" t="n"/>
-      <c r="E34" s="16" t="n"/>
-      <c r="F34" s="18" t="n"/>
-      <c r="G34" s="18" t="n"/>
-      <c r="H34" s="17" t="n"/>
-    </row>
-    <row r="35" ht="27" customHeight="1">
-      <c r="A35" s="16" t="n"/>
-      <c r="B35" s="17" t="n"/>
-      <c r="C35" s="17" t="n"/>
-      <c r="D35" s="16" t="n"/>
-      <c r="E35" s="16" t="n"/>
-      <c r="F35" s="18" t="n"/>
-      <c r="G35" s="18" t="n"/>
-      <c r="H35" s="17" t="n"/>
-    </row>
-    <row r="36" ht="27" customHeight="1">
+    <row r="36" ht="20" customHeight="1">
       <c r="A36" s="16" t="n"/>
       <c r="B36" s="17" t="n"/>
       <c r="C36" s="17" t="n"/>
@@ -1018,7 +912,7 @@
       <c r="G36" s="18" t="n"/>
       <c r="H36" s="17" t="n"/>
     </row>
-    <row r="37" ht="27" customHeight="1">
+    <row r="37" ht="20" customHeight="1">
       <c r="A37" s="16" t="n"/>
       <c r="B37" s="17" t="n"/>
       <c r="C37" s="17" t="n"/>
@@ -1028,7 +922,7 @@
       <c r="G37" s="18" t="n"/>
       <c r="H37" s="17" t="n"/>
     </row>
-    <row r="38" ht="27" customHeight="1">
+    <row r="38" ht="20" customHeight="1">
       <c r="A38" s="16" t="n"/>
       <c r="B38" s="17" t="n"/>
       <c r="C38" s="17" t="n"/>
@@ -1038,7 +932,7 @@
       <c r="G38" s="18" t="n"/>
       <c r="H38" s="17" t="n"/>
     </row>
-    <row r="39" ht="27" customHeight="1">
+    <row r="39" ht="20" customHeight="1">
       <c r="A39" s="16" t="n"/>
       <c r="B39" s="17" t="n"/>
       <c r="C39" s="17" t="n"/>
@@ -1048,7 +942,7 @@
       <c r="G39" s="18" t="n"/>
       <c r="H39" s="17" t="n"/>
     </row>
-    <row r="40" ht="27" customHeight="1">
+    <row r="40" ht="20" customHeight="1">
       <c r="A40" s="16" t="n"/>
       <c r="B40" s="17" t="n"/>
       <c r="C40" s="17" t="n"/>
@@ -1058,7 +952,7 @@
       <c r="G40" s="18" t="n"/>
       <c r="H40" s="17" t="n"/>
     </row>
-    <row r="41" ht="27" customHeight="1">
+    <row r="41" ht="20" customHeight="1">
       <c r="A41" s="16" t="n"/>
       <c r="B41" s="17" t="n"/>
       <c r="C41" s="17" t="n"/>
@@ -1068,7 +962,7 @@
       <c r="G41" s="18" t="n"/>
       <c r="H41" s="17" t="n"/>
     </row>
-    <row r="42" ht="27" customHeight="1">
+    <row r="42" ht="20" customHeight="1">
       <c r="A42" s="16" t="n"/>
       <c r="B42" s="17" t="n"/>
       <c r="C42" s="17" t="n"/>
@@ -1078,7 +972,7 @@
       <c r="G42" s="18" t="n"/>
       <c r="H42" s="17" t="n"/>
     </row>
-    <row r="43" ht="27" customHeight="1">
+    <row r="43" ht="20" customHeight="1">
       <c r="A43" s="16" t="n"/>
       <c r="B43" s="17" t="n"/>
       <c r="C43" s="17" t="n"/>
@@ -1088,7 +982,7 @@
       <c r="G43" s="18" t="n"/>
       <c r="H43" s="17" t="n"/>
     </row>
-    <row r="44" ht="27" customHeight="1">
+    <row r="44" ht="20" customHeight="1">
       <c r="A44" s="16" t="n"/>
       <c r="B44" s="17" t="n"/>
       <c r="C44" s="17" t="n"/>
@@ -1098,7 +992,7 @@
       <c r="G44" s="18" t="n"/>
       <c r="H44" s="17" t="n"/>
     </row>
-    <row r="45" ht="27" customHeight="1">
+    <row r="45" ht="20" customHeight="1">
       <c r="A45" s="16" t="n"/>
       <c r="B45" s="17" t="n"/>
       <c r="C45" s="17" t="n"/>
@@ -1108,7 +1002,7 @@
       <c r="G45" s="18" t="n"/>
       <c r="H45" s="17" t="n"/>
     </row>
-    <row r="46" ht="27" customHeight="1">
+    <row r="46" ht="20" customHeight="1">
       <c r="A46" s="16" t="n"/>
       <c r="B46" s="17" t="n"/>
       <c r="C46" s="17" t="n"/>
@@ -1118,7 +1012,7 @@
       <c r="G46" s="18" t="n"/>
       <c r="H46" s="17" t="n"/>
     </row>
-    <row r="47" ht="27" customHeight="1">
+    <row r="47" ht="20" customHeight="1">
       <c r="A47" s="16" t="n"/>
       <c r="B47" s="17" t="n"/>
       <c r="C47" s="17" t="n"/>
@@ -1128,7 +1022,7 @@
       <c r="G47" s="18" t="n"/>
       <c r="H47" s="17" t="n"/>
     </row>
-    <row r="48" ht="27" customHeight="1">
+    <row r="48" ht="20" customHeight="1">
       <c r="A48" s="16" t="n"/>
       <c r="B48" s="17" t="n"/>
       <c r="C48" s="17" t="n"/>
@@ -1138,7 +1032,7 @@
       <c r="G48" s="18" t="n"/>
       <c r="H48" s="17" t="n"/>
     </row>
-    <row r="49" ht="27" customHeight="1">
+    <row r="49" ht="20" customHeight="1">
       <c r="A49" s="16" t="n"/>
       <c r="B49" s="17" t="n"/>
       <c r="C49" s="17" t="n"/>
@@ -1148,7 +1042,7 @@
       <c r="G49" s="18" t="n"/>
       <c r="H49" s="17" t="n"/>
     </row>
-    <row r="50" ht="27" customHeight="1">
+    <row r="50" ht="20" customHeight="1">
       <c r="A50" s="16" t="n"/>
       <c r="B50" s="17" t="n"/>
       <c r="C50" s="17" t="n"/>
@@ -1158,7 +1052,7 @@
       <c r="G50" s="18" t="n"/>
       <c r="H50" s="17" t="n"/>
     </row>
-    <row r="51" ht="27" customHeight="1">
+    <row r="51" ht="20" customHeight="1">
       <c r="A51" s="16" t="n"/>
       <c r="B51" s="17" t="n"/>
       <c r="C51" s="17" t="n"/>
@@ -1168,127 +1062,104 @@
       <c r="G51" s="18" t="n"/>
       <c r="H51" s="17" t="n"/>
     </row>
-    <row r="52" ht="27" customHeight="1">
-      <c r="A52" s="16" t="n"/>
-      <c r="B52" s="17" t="n"/>
-      <c r="C52" s="17" t="n"/>
-      <c r="D52" s="16" t="n"/>
-      <c r="E52" s="16" t="n"/>
-      <c r="F52" s="18" t="n"/>
-      <c r="G52" s="18" t="n"/>
-      <c r="H52" s="17" t="n"/>
-    </row>
-    <row r="53" ht="27" customHeight="1">
-      <c r="A53" s="16" t="n"/>
-      <c r="B53" s="17" t="n"/>
-      <c r="C53" s="17" t="n"/>
-      <c r="D53" s="16" t="n"/>
-      <c r="E53" s="16" t="n"/>
-      <c r="F53" s="18" t="n"/>
-      <c r="G53" s="18" t="n"/>
-      <c r="H53" s="17" t="n"/>
-    </row>
-    <row r="54" ht="27" customHeight="1">
-      <c r="A54" s="16" t="n"/>
-      <c r="B54" s="17" t="n"/>
-      <c r="C54" s="17" t="n"/>
-      <c r="D54" s="16" t="n"/>
-      <c r="E54" s="16" t="n"/>
-      <c r="F54" s="18" t="n"/>
-      <c r="G54" s="18" t="n"/>
-      <c r="H54" s="17" t="n"/>
-    </row>
-    <row r="55" ht="27" customHeight="1">
-      <c r="A55" s="16" t="n"/>
-      <c r="B55" s="17" t="n"/>
-      <c r="C55" s="17" t="n"/>
-      <c r="D55" s="16" t="n"/>
-      <c r="E55" s="16" t="n"/>
-      <c r="F55" s="18" t="n"/>
-      <c r="G55" s="18" t="n"/>
-      <c r="H55" s="17" t="n"/>
-    </row>
-    <row r="56" ht="27" customHeight="1">
-      <c r="A56" s="16" t="n"/>
-      <c r="B56" s="17" t="n"/>
-      <c r="C56" s="17" t="n"/>
-      <c r="D56" s="16" t="n"/>
-      <c r="E56" s="16" t="n"/>
-      <c r="F56" s="18" t="n"/>
-      <c r="G56" s="18" t="n"/>
-      <c r="H56" s="17" t="n"/>
-    </row>
-    <row r="57" ht="27" customHeight="1">
-      <c r="A57" s="16" t="n"/>
-      <c r="B57" s="17" t="n"/>
-      <c r="C57" s="17" t="n"/>
-      <c r="D57" s="16" t="n"/>
-      <c r="E57" s="16" t="n"/>
-      <c r="F57" s="18" t="n"/>
-      <c r="G57" s="18" t="n"/>
-      <c r="H57" s="17" t="n"/>
-    </row>
-    <row r="58" ht="27" customHeight="1">
-      <c r="A58" s="16" t="n"/>
-      <c r="B58" s="17" t="n"/>
-      <c r="C58" s="17" t="n"/>
-      <c r="D58" s="16" t="n"/>
-      <c r="E58" s="16" t="n"/>
-      <c r="F58" s="18" t="n"/>
-      <c r="G58" s="18" t="n"/>
-      <c r="H58" s="17" t="n"/>
-    </row>
-    <row r="59" ht="27" customHeight="1">
-      <c r="A59" s="16" t="n"/>
-      <c r="B59" s="17" t="n"/>
-      <c r="C59" s="17" t="n"/>
-      <c r="D59" s="16" t="n"/>
-      <c r="E59" s="16" t="n"/>
-      <c r="F59" s="18" t="n"/>
-      <c r="G59" s="18" t="n"/>
-      <c r="H59" s="17" t="n"/>
-    </row>
-    <row r="60" ht="27" customHeight="1">
-      <c r="A60" s="16" t="n"/>
-      <c r="B60" s="17" t="n"/>
-      <c r="C60" s="17" t="n"/>
-      <c r="D60" s="16" t="n"/>
-      <c r="E60" s="16" t="n"/>
-      <c r="F60" s="18" t="n"/>
-      <c r="G60" s="18" t="n"/>
-      <c r="H60" s="17" t="n"/>
-    </row>
-    <row r="61" ht="27" customHeight="1">
-      <c r="A61" s="16" t="n"/>
-      <c r="B61" s="17" t="n"/>
-      <c r="C61" s="17" t="n"/>
-      <c r="D61" s="16" t="n"/>
-      <c r="E61" s="16" t="n"/>
-      <c r="F61" s="18" t="n"/>
-      <c r="G61" s="18" t="n"/>
-      <c r="H61" s="17" t="n"/>
-    </row>
-    <row r="62" ht="27" customHeight="1">
-      <c r="A62" s="16" t="n"/>
-      <c r="B62" s="17" t="n"/>
-      <c r="C62" s="17" t="n"/>
-      <c r="D62" s="16" t="n"/>
-      <c r="E62" s="16" t="n"/>
-      <c r="F62" s="18" t="n"/>
-      <c r="G62" s="18" t="n"/>
-      <c r="H62" s="17" t="n"/>
-    </row>
-    <row r="63" ht="27" customHeight="1">
-      <c r="A63" s="16" t="n"/>
-      <c r="B63" s="17" t="n"/>
-      <c r="C63" s="17" t="n"/>
-      <c r="D63" s="16" t="n"/>
-      <c r="E63" s="16" t="n"/>
-      <c r="F63" s="18" t="n"/>
-      <c r="G63" s="18" t="n"/>
-      <c r="H63" s="17" t="n"/>
-    </row>
-    <row r="64" ht="27" customHeight="1">
+    <row r="53">
+      <c r="A53" s="19" t="inlineStr">
+        <is>
+          <t>※工事内容明細には消費税が含まれておりません。</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="19" customHeight="1">
+      <c r="E55" s="20" t="inlineStr">
+        <is>
+          <t>小　　計</t>
+        </is>
+      </c>
+      <c r="G55" s="21" t="n"/>
+    </row>
+    <row r="56" ht="19" customHeight="1">
+      <c r="E56" s="20" t="inlineStr">
+        <is>
+          <t>値 引 き</t>
+        </is>
+      </c>
+      <c r="G56" s="21" t="n"/>
+    </row>
+    <row r="57" ht="19" customHeight="1">
+      <c r="E57" s="20" t="inlineStr">
+        <is>
+          <t>税抜合計</t>
+        </is>
+      </c>
+      <c r="G57" s="21" t="n"/>
+    </row>
+    <row r="58" ht="19" customHeight="1">
+      <c r="E58" s="20" t="inlineStr">
+        <is>
+          <t>消 費 税</t>
+        </is>
+      </c>
+      <c r="G58" s="21" t="n"/>
+    </row>
+    <row r="59" ht="22" customHeight="1">
+      <c r="E59" s="22" t="inlineStr">
+        <is>
+          <t>税込合計</t>
+        </is>
+      </c>
+      <c r="G59" s="23" t="n"/>
+    </row>
+    <row r="60" ht="12" customHeight="1"/>
+    <row r="62" ht="22" customHeight="1">
+      <c r="A62" s="24" t="inlineStr">
+        <is>
+          <t>工 事 内 容 明 細</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="22" customHeight="1">
+      <c r="A63" s="15" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="B63" s="15" t="inlineStr">
+        <is>
+          <t>工事品目</t>
+        </is>
+      </c>
+      <c r="C63" s="15" t="inlineStr">
+        <is>
+          <t>仕様</t>
+        </is>
+      </c>
+      <c r="D63" s="15" t="inlineStr">
+        <is>
+          <t>数量</t>
+        </is>
+      </c>
+      <c r="E63" s="15" t="inlineStr">
+        <is>
+          <t>単位</t>
+        </is>
+      </c>
+      <c r="F63" s="15" t="inlineStr">
+        <is>
+          <t>単価</t>
+        </is>
+      </c>
+      <c r="G63" s="15" t="inlineStr">
+        <is>
+          <t>金額</t>
+        </is>
+      </c>
+      <c r="H63" s="15" t="inlineStr">
+        <is>
+          <t>備考</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="19" customHeight="1">
       <c r="A64" s="16" t="n"/>
       <c r="B64" s="17" t="n"/>
       <c r="C64" s="17" t="n"/>
@@ -1298,7 +1169,7 @@
       <c r="G64" s="18" t="n"/>
       <c r="H64" s="17" t="n"/>
     </row>
-    <row r="65" ht="27" customHeight="1">
+    <row r="65" ht="19" customHeight="1">
       <c r="A65" s="16" t="n"/>
       <c r="B65" s="17" t="n"/>
       <c r="C65" s="17" t="n"/>
@@ -1308,7 +1179,7 @@
       <c r="G65" s="18" t="n"/>
       <c r="H65" s="17" t="n"/>
     </row>
-    <row r="66" ht="27" customHeight="1">
+    <row r="66" ht="19" customHeight="1">
       <c r="A66" s="16" t="n"/>
       <c r="B66" s="17" t="n"/>
       <c r="C66" s="17" t="n"/>
@@ -1318,7 +1189,7 @@
       <c r="G66" s="18" t="n"/>
       <c r="H66" s="17" t="n"/>
     </row>
-    <row r="67" ht="27" customHeight="1">
+    <row r="67" ht="19" customHeight="1">
       <c r="A67" s="16" t="n"/>
       <c r="B67" s="17" t="n"/>
       <c r="C67" s="17" t="n"/>
@@ -1328,7 +1199,7 @@
       <c r="G67" s="18" t="n"/>
       <c r="H67" s="17" t="n"/>
     </row>
-    <row r="68" ht="27" customHeight="1">
+    <row r="68" ht="19" customHeight="1">
       <c r="A68" s="16" t="n"/>
       <c r="B68" s="17" t="n"/>
       <c r="C68" s="17" t="n"/>
@@ -1338,7 +1209,7 @@
       <c r="G68" s="18" t="n"/>
       <c r="H68" s="17" t="n"/>
     </row>
-    <row r="69" ht="27" customHeight="1">
+    <row r="69" ht="19" customHeight="1">
       <c r="A69" s="16" t="n"/>
       <c r="B69" s="17" t="n"/>
       <c r="C69" s="17" t="n"/>
@@ -1348,7 +1219,7 @@
       <c r="G69" s="18" t="n"/>
       <c r="H69" s="17" t="n"/>
     </row>
-    <row r="70" ht="27" customHeight="1">
+    <row r="70" ht="19" customHeight="1">
       <c r="A70" s="16" t="n"/>
       <c r="B70" s="17" t="n"/>
       <c r="C70" s="17" t="n"/>
@@ -1358,7 +1229,7 @@
       <c r="G70" s="18" t="n"/>
       <c r="H70" s="17" t="n"/>
     </row>
-    <row r="71" ht="27" customHeight="1">
+    <row r="71" ht="19" customHeight="1">
       <c r="A71" s="16" t="n"/>
       <c r="B71" s="17" t="n"/>
       <c r="C71" s="17" t="n"/>
@@ -1368,7 +1239,7 @@
       <c r="G71" s="18" t="n"/>
       <c r="H71" s="17" t="n"/>
     </row>
-    <row r="72" ht="27" customHeight="1">
+    <row r="72" ht="19" customHeight="1">
       <c r="A72" s="16" t="n"/>
       <c r="B72" s="17" t="n"/>
       <c r="C72" s="17" t="n"/>
@@ -1378,7 +1249,7 @@
       <c r="G72" s="18" t="n"/>
       <c r="H72" s="17" t="n"/>
     </row>
-    <row r="73" ht="27" customHeight="1">
+    <row r="73" ht="19" customHeight="1">
       <c r="A73" s="16" t="n"/>
       <c r="B73" s="17" t="n"/>
       <c r="C73" s="17" t="n"/>
@@ -1388,7 +1259,7 @@
       <c r="G73" s="18" t="n"/>
       <c r="H73" s="17" t="n"/>
     </row>
-    <row r="74" ht="27" customHeight="1">
+    <row r="74" ht="19" customHeight="1">
       <c r="A74" s="16" t="n"/>
       <c r="B74" s="17" t="n"/>
       <c r="C74" s="17" t="n"/>
@@ -1398,7 +1269,7 @@
       <c r="G74" s="18" t="n"/>
       <c r="H74" s="17" t="n"/>
     </row>
-    <row r="75" ht="27" customHeight="1">
+    <row r="75" ht="19" customHeight="1">
       <c r="A75" s="16" t="n"/>
       <c r="B75" s="17" t="n"/>
       <c r="C75" s="17" t="n"/>
@@ -1408,7 +1279,7 @@
       <c r="G75" s="18" t="n"/>
       <c r="H75" s="17" t="n"/>
     </row>
-    <row r="76" ht="27" customHeight="1">
+    <row r="76" ht="19" customHeight="1">
       <c r="A76" s="16" t="n"/>
       <c r="B76" s="17" t="n"/>
       <c r="C76" s="17" t="n"/>
@@ -1418,7 +1289,7 @@
       <c r="G76" s="18" t="n"/>
       <c r="H76" s="17" t="n"/>
     </row>
-    <row r="77" ht="27" customHeight="1">
+    <row r="77" ht="19" customHeight="1">
       <c r="A77" s="16" t="n"/>
       <c r="B77" s="17" t="n"/>
       <c r="C77" s="17" t="n"/>
@@ -1428,7 +1299,7 @@
       <c r="G77" s="18" t="n"/>
       <c r="H77" s="17" t="n"/>
     </row>
-    <row r="78" ht="27" customHeight="1">
+    <row r="78" ht="19" customHeight="1">
       <c r="A78" s="16" t="n"/>
       <c r="B78" s="17" t="n"/>
       <c r="C78" s="17" t="n"/>
@@ -1438,7 +1309,7 @@
       <c r="G78" s="18" t="n"/>
       <c r="H78" s="17" t="n"/>
     </row>
-    <row r="79" ht="27" customHeight="1">
+    <row r="79" ht="19" customHeight="1">
       <c r="A79" s="16" t="n"/>
       <c r="B79" s="17" t="n"/>
       <c r="C79" s="17" t="n"/>
@@ -1448,7 +1319,7 @@
       <c r="G79" s="18" t="n"/>
       <c r="H79" s="17" t="n"/>
     </row>
-    <row r="80" ht="27" customHeight="1">
+    <row r="80" ht="19" customHeight="1">
       <c r="A80" s="16" t="n"/>
       <c r="B80" s="17" t="n"/>
       <c r="C80" s="17" t="n"/>
@@ -1458,7 +1329,7 @@
       <c r="G80" s="18" t="n"/>
       <c r="H80" s="17" t="n"/>
     </row>
-    <row r="81" ht="27" customHeight="1">
+    <row r="81" ht="19" customHeight="1">
       <c r="A81" s="16" t="n"/>
       <c r="B81" s="17" t="n"/>
       <c r="C81" s="17" t="n"/>
@@ -1468,7 +1339,7 @@
       <c r="G81" s="18" t="n"/>
       <c r="H81" s="17" t="n"/>
     </row>
-    <row r="82" ht="27" customHeight="1">
+    <row r="82" ht="19" customHeight="1">
       <c r="A82" s="16" t="n"/>
       <c r="B82" s="17" t="n"/>
       <c r="C82" s="17" t="n"/>
@@ -1478,7 +1349,7 @@
       <c r="G82" s="18" t="n"/>
       <c r="H82" s="17" t="n"/>
     </row>
-    <row r="83" ht="27" customHeight="1">
+    <row r="83" ht="19" customHeight="1">
       <c r="A83" s="16" t="n"/>
       <c r="B83" s="17" t="n"/>
       <c r="C83" s="17" t="n"/>
@@ -1488,47 +1359,77 @@
       <c r="G83" s="18" t="n"/>
       <c r="H83" s="17" t="n"/>
     </row>
-    <row r="84" ht="27" customHeight="1">
-      <c r="A84" s="16" t="n"/>
-      <c r="B84" s="17" t="n"/>
-      <c r="C84" s="17" t="n"/>
-      <c r="D84" s="16" t="n"/>
-      <c r="E84" s="16" t="n"/>
-      <c r="F84" s="18" t="n"/>
-      <c r="G84" s="18" t="n"/>
-      <c r="H84" s="17" t="n"/>
-    </row>
-    <row r="85" ht="27" customHeight="1">
-      <c r="A85" s="16" t="n"/>
-      <c r="B85" s="17" t="n"/>
-      <c r="C85" s="17" t="n"/>
-      <c r="D85" s="16" t="n"/>
-      <c r="E85" s="16" t="n"/>
-      <c r="F85" s="18" t="n"/>
-      <c r="G85" s="18" t="n"/>
-      <c r="H85" s="17" t="n"/>
-    </row>
-    <row r="86" ht="27" customHeight="1">
-      <c r="A86" s="16" t="n"/>
-      <c r="B86" s="17" t="n"/>
-      <c r="C86" s="17" t="n"/>
-      <c r="D86" s="16" t="n"/>
-      <c r="E86" s="16" t="n"/>
-      <c r="F86" s="18" t="n"/>
-      <c r="G86" s="18" t="n"/>
-      <c r="H86" s="17" t="n"/>
-    </row>
-    <row r="87" ht="27" customHeight="1">
-      <c r="A87" s="16" t="n"/>
-      <c r="B87" s="17" t="n"/>
-      <c r="C87" s="17" t="n"/>
-      <c r="D87" s="16" t="n"/>
-      <c r="E87" s="16" t="n"/>
-      <c r="F87" s="18" t="n"/>
-      <c r="G87" s="18" t="n"/>
-      <c r="H87" s="17" t="n"/>
-    </row>
-    <row r="88" ht="27" customHeight="1">
+    <row r="84" ht="18" customHeight="1">
+      <c r="A84" s="25" t="inlineStr">
+        <is>
+          <t>※工事内容明細には消費税が含まれておりません。</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="22" customHeight="1">
+      <c r="A85" s="26" t="n"/>
+      <c r="B85" s="26" t="n"/>
+      <c r="C85" s="26" t="n"/>
+      <c r="D85" s="26" t="n"/>
+      <c r="E85" s="26" t="n"/>
+      <c r="F85" s="27" t="inlineStr">
+        <is>
+          <t>合　計</t>
+        </is>
+      </c>
+      <c r="G85" s="28" t="n"/>
+      <c r="H85" s="26" t="n"/>
+    </row>
+    <row r="86" ht="22" customHeight="1">
+      <c r="A86" s="24" t="inlineStr">
+        <is>
+          <t>工 事 内 容 明 細</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="22" customHeight="1">
+      <c r="A87" s="15" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="B87" s="15" t="inlineStr">
+        <is>
+          <t>工事品目</t>
+        </is>
+      </c>
+      <c r="C87" s="15" t="inlineStr">
+        <is>
+          <t>仕様</t>
+        </is>
+      </c>
+      <c r="D87" s="15" t="inlineStr">
+        <is>
+          <t>数量</t>
+        </is>
+      </c>
+      <c r="E87" s="15" t="inlineStr">
+        <is>
+          <t>単位</t>
+        </is>
+      </c>
+      <c r="F87" s="15" t="inlineStr">
+        <is>
+          <t>単価</t>
+        </is>
+      </c>
+      <c r="G87" s="15" t="inlineStr">
+        <is>
+          <t>金額</t>
+        </is>
+      </c>
+      <c r="H87" s="15" t="inlineStr">
+        <is>
+          <t>備考</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="19" customHeight="1">
       <c r="A88" s="16" t="n"/>
       <c r="B88" s="17" t="n"/>
       <c r="C88" s="17" t="n"/>
@@ -1538,7 +1439,7 @@
       <c r="G88" s="18" t="n"/>
       <c r="H88" s="17" t="n"/>
     </row>
-    <row r="89" ht="27" customHeight="1">
+    <row r="89" ht="19" customHeight="1">
       <c r="A89" s="16" t="n"/>
       <c r="B89" s="17" t="n"/>
       <c r="C89" s="17" t="n"/>
@@ -1548,7 +1449,7 @@
       <c r="G89" s="18" t="n"/>
       <c r="H89" s="17" t="n"/>
     </row>
-    <row r="90" ht="27" customHeight="1">
+    <row r="90" ht="19" customHeight="1">
       <c r="A90" s="16" t="n"/>
       <c r="B90" s="17" t="n"/>
       <c r="C90" s="17" t="n"/>
@@ -1558,7 +1459,7 @@
       <c r="G90" s="18" t="n"/>
       <c r="H90" s="17" t="n"/>
     </row>
-    <row r="91" ht="27" customHeight="1">
+    <row r="91" ht="19" customHeight="1">
       <c r="A91" s="16" t="n"/>
       <c r="B91" s="17" t="n"/>
       <c r="C91" s="17" t="n"/>
@@ -1568,7 +1469,7 @@
       <c r="G91" s="18" t="n"/>
       <c r="H91" s="17" t="n"/>
     </row>
-    <row r="92" ht="27" customHeight="1">
+    <row r="92" ht="19" customHeight="1">
       <c r="A92" s="16" t="n"/>
       <c r="B92" s="17" t="n"/>
       <c r="C92" s="17" t="n"/>
@@ -1578,7 +1479,7 @@
       <c r="G92" s="18" t="n"/>
       <c r="H92" s="17" t="n"/>
     </row>
-    <row r="93" ht="27" customHeight="1">
+    <row r="93" ht="19" customHeight="1">
       <c r="A93" s="16" t="n"/>
       <c r="B93" s="17" t="n"/>
       <c r="C93" s="17" t="n"/>
@@ -1588,7 +1489,7 @@
       <c r="G93" s="18" t="n"/>
       <c r="H93" s="17" t="n"/>
     </row>
-    <row r="94" ht="27" customHeight="1">
+    <row r="94" ht="19" customHeight="1">
       <c r="A94" s="16" t="n"/>
       <c r="B94" s="17" t="n"/>
       <c r="C94" s="17" t="n"/>
@@ -1598,7 +1499,7 @@
       <c r="G94" s="18" t="n"/>
       <c r="H94" s="17" t="n"/>
     </row>
-    <row r="95" ht="27" customHeight="1">
+    <row r="95" ht="19" customHeight="1">
       <c r="A95" s="16" t="n"/>
       <c r="B95" s="17" t="n"/>
       <c r="C95" s="17" t="n"/>
@@ -1608,7 +1509,7 @@
       <c r="G95" s="18" t="n"/>
       <c r="H95" s="17" t="n"/>
     </row>
-    <row r="96" ht="27" customHeight="1">
+    <row r="96" ht="19" customHeight="1">
       <c r="A96" s="16" t="n"/>
       <c r="B96" s="17" t="n"/>
       <c r="C96" s="17" t="n"/>
@@ -1618,7 +1519,7 @@
       <c r="G96" s="18" t="n"/>
       <c r="H96" s="17" t="n"/>
     </row>
-    <row r="97" ht="27" customHeight="1">
+    <row r="97" ht="19" customHeight="1">
       <c r="A97" s="16" t="n"/>
       <c r="B97" s="17" t="n"/>
       <c r="C97" s="17" t="n"/>
@@ -1628,7 +1529,7 @@
       <c r="G97" s="18" t="n"/>
       <c r="H97" s="17" t="n"/>
     </row>
-    <row r="98" ht="27" customHeight="1">
+    <row r="98" ht="19" customHeight="1">
       <c r="A98" s="16" t="n"/>
       <c r="B98" s="17" t="n"/>
       <c r="C98" s="17" t="n"/>
@@ -1638,7 +1539,7 @@
       <c r="G98" s="18" t="n"/>
       <c r="H98" s="17" t="n"/>
     </row>
-    <row r="99" ht="27" customHeight="1">
+    <row r="99" ht="19" customHeight="1">
       <c r="A99" s="16" t="n"/>
       <c r="B99" s="17" t="n"/>
       <c r="C99" s="17" t="n"/>
@@ -1648,7 +1549,7 @@
       <c r="G99" s="18" t="n"/>
       <c r="H99" s="17" t="n"/>
     </row>
-    <row r="100" ht="27" customHeight="1">
+    <row r="100" ht="19" customHeight="1">
       <c r="A100" s="16" t="n"/>
       <c r="B100" s="17" t="n"/>
       <c r="C100" s="17" t="n"/>
@@ -1658,7 +1559,7 @@
       <c r="G100" s="18" t="n"/>
       <c r="H100" s="17" t="n"/>
     </row>
-    <row r="101" ht="27" customHeight="1">
+    <row r="101" ht="19" customHeight="1">
       <c r="A101" s="16" t="n"/>
       <c r="B101" s="17" t="n"/>
       <c r="C101" s="17" t="n"/>
@@ -1668,7 +1569,7 @@
       <c r="G101" s="18" t="n"/>
       <c r="H101" s="17" t="n"/>
     </row>
-    <row r="102" ht="27" customHeight="1">
+    <row r="102" ht="19" customHeight="1">
       <c r="A102" s="16" t="n"/>
       <c r="B102" s="17" t="n"/>
       <c r="C102" s="17" t="n"/>
@@ -1678,7 +1579,7 @@
       <c r="G102" s="18" t="n"/>
       <c r="H102" s="17" t="n"/>
     </row>
-    <row r="103" ht="27" customHeight="1">
+    <row r="103" ht="19" customHeight="1">
       <c r="A103" s="16" t="n"/>
       <c r="B103" s="17" t="n"/>
       <c r="C103" s="17" t="n"/>
@@ -1688,7 +1589,7 @@
       <c r="G103" s="18" t="n"/>
       <c r="H103" s="17" t="n"/>
     </row>
-    <row r="104" ht="27" customHeight="1">
+    <row r="104" ht="19" customHeight="1">
       <c r="A104" s="16" t="n"/>
       <c r="B104" s="17" t="n"/>
       <c r="C104" s="17" t="n"/>
@@ -1698,7 +1599,7 @@
       <c r="G104" s="18" t="n"/>
       <c r="H104" s="17" t="n"/>
     </row>
-    <row r="105" ht="27" customHeight="1">
+    <row r="105" ht="19" customHeight="1">
       <c r="A105" s="16" t="n"/>
       <c r="B105" s="17" t="n"/>
       <c r="C105" s="17" t="n"/>
@@ -1708,7 +1609,7 @@
       <c r="G105" s="18" t="n"/>
       <c r="H105" s="17" t="n"/>
     </row>
-    <row r="106" ht="27" customHeight="1">
+    <row r="106" ht="19" customHeight="1">
       <c r="A106" s="16" t="n"/>
       <c r="B106" s="17" t="n"/>
       <c r="C106" s="17" t="n"/>
@@ -1718,7 +1619,7 @@
       <c r="G106" s="18" t="n"/>
       <c r="H106" s="17" t="n"/>
     </row>
-    <row r="107" ht="27" customHeight="1">
+    <row r="107" ht="19" customHeight="1">
       <c r="A107" s="16" t="n"/>
       <c r="B107" s="17" t="n"/>
       <c r="C107" s="17" t="n"/>
@@ -1728,47 +1629,77 @@
       <c r="G107" s="18" t="n"/>
       <c r="H107" s="17" t="n"/>
     </row>
-    <row r="108" ht="27" customHeight="1">
-      <c r="A108" s="16" t="n"/>
-      <c r="B108" s="17" t="n"/>
-      <c r="C108" s="17" t="n"/>
-      <c r="D108" s="16" t="n"/>
-      <c r="E108" s="16" t="n"/>
-      <c r="F108" s="18" t="n"/>
-      <c r="G108" s="18" t="n"/>
-      <c r="H108" s="17" t="n"/>
-    </row>
-    <row r="109" ht="27" customHeight="1">
-      <c r="A109" s="16" t="n"/>
-      <c r="B109" s="17" t="n"/>
-      <c r="C109" s="17" t="n"/>
-      <c r="D109" s="16" t="n"/>
-      <c r="E109" s="16" t="n"/>
-      <c r="F109" s="18" t="n"/>
-      <c r="G109" s="18" t="n"/>
-      <c r="H109" s="17" t="n"/>
-    </row>
-    <row r="110" ht="27" customHeight="1">
-      <c r="A110" s="16" t="n"/>
-      <c r="B110" s="17" t="n"/>
-      <c r="C110" s="17" t="n"/>
-      <c r="D110" s="16" t="n"/>
-      <c r="E110" s="16" t="n"/>
-      <c r="F110" s="18" t="n"/>
-      <c r="G110" s="18" t="n"/>
-      <c r="H110" s="17" t="n"/>
-    </row>
-    <row r="111" ht="27" customHeight="1">
-      <c r="A111" s="16" t="n"/>
-      <c r="B111" s="17" t="n"/>
-      <c r="C111" s="17" t="n"/>
-      <c r="D111" s="16" t="n"/>
-      <c r="E111" s="16" t="n"/>
-      <c r="F111" s="18" t="n"/>
-      <c r="G111" s="18" t="n"/>
-      <c r="H111" s="17" t="n"/>
-    </row>
-    <row r="112" ht="27" customHeight="1">
+    <row r="108" ht="18" customHeight="1">
+      <c r="A108" s="25" t="inlineStr">
+        <is>
+          <t>※工事内容明細には消費税が含まれておりません。</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="22" customHeight="1">
+      <c r="A109" s="26" t="n"/>
+      <c r="B109" s="26" t="n"/>
+      <c r="C109" s="26" t="n"/>
+      <c r="D109" s="26" t="n"/>
+      <c r="E109" s="26" t="n"/>
+      <c r="F109" s="27" t="inlineStr">
+        <is>
+          <t>合　計</t>
+        </is>
+      </c>
+      <c r="G109" s="28" t="n"/>
+      <c r="H109" s="26" t="n"/>
+    </row>
+    <row r="110" ht="22" customHeight="1">
+      <c r="A110" s="24" t="inlineStr">
+        <is>
+          <t>工 事 内 容 明 細</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="22" customHeight="1">
+      <c r="A111" s="15" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="B111" s="15" t="inlineStr">
+        <is>
+          <t>工事品目</t>
+        </is>
+      </c>
+      <c r="C111" s="15" t="inlineStr">
+        <is>
+          <t>仕様</t>
+        </is>
+      </c>
+      <c r="D111" s="15" t="inlineStr">
+        <is>
+          <t>数量</t>
+        </is>
+      </c>
+      <c r="E111" s="15" t="inlineStr">
+        <is>
+          <t>単位</t>
+        </is>
+      </c>
+      <c r="F111" s="15" t="inlineStr">
+        <is>
+          <t>単価</t>
+        </is>
+      </c>
+      <c r="G111" s="15" t="inlineStr">
+        <is>
+          <t>金額</t>
+        </is>
+      </c>
+      <c r="H111" s="15" t="inlineStr">
+        <is>
+          <t>備考</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="19" customHeight="1">
       <c r="A112" s="16" t="n"/>
       <c r="B112" s="17" t="n"/>
       <c r="C112" s="17" t="n"/>
@@ -1778,7 +1709,7 @@
       <c r="G112" s="18" t="n"/>
       <c r="H112" s="17" t="n"/>
     </row>
-    <row r="113" ht="27" customHeight="1">
+    <row r="113" ht="19" customHeight="1">
       <c r="A113" s="16" t="n"/>
       <c r="B113" s="17" t="n"/>
       <c r="C113" s="17" t="n"/>
@@ -1788,7 +1719,7 @@
       <c r="G113" s="18" t="n"/>
       <c r="H113" s="17" t="n"/>
     </row>
-    <row r="114" ht="27" customHeight="1">
+    <row r="114" ht="19" customHeight="1">
       <c r="A114" s="16" t="n"/>
       <c r="B114" s="17" t="n"/>
       <c r="C114" s="17" t="n"/>
@@ -1798,7 +1729,7 @@
       <c r="G114" s="18" t="n"/>
       <c r="H114" s="17" t="n"/>
     </row>
-    <row r="115" ht="27" customHeight="1">
+    <row r="115" ht="19" customHeight="1">
       <c r="A115" s="16" t="n"/>
       <c r="B115" s="17" t="n"/>
       <c r="C115" s="17" t="n"/>
@@ -1808,7 +1739,7 @@
       <c r="G115" s="18" t="n"/>
       <c r="H115" s="17" t="n"/>
     </row>
-    <row r="116" ht="27" customHeight="1">
+    <row r="116" ht="19" customHeight="1">
       <c r="A116" s="16" t="n"/>
       <c r="B116" s="17" t="n"/>
       <c r="C116" s="17" t="n"/>
@@ -1818,7 +1749,7 @@
       <c r="G116" s="18" t="n"/>
       <c r="H116" s="17" t="n"/>
     </row>
-    <row r="117" ht="27" customHeight="1">
+    <row r="117" ht="19" customHeight="1">
       <c r="A117" s="16" t="n"/>
       <c r="B117" s="17" t="n"/>
       <c r="C117" s="17" t="n"/>
@@ -1828,7 +1759,7 @@
       <c r="G117" s="18" t="n"/>
       <c r="H117" s="17" t="n"/>
     </row>
-    <row r="118" ht="27" customHeight="1">
+    <row r="118" ht="19" customHeight="1">
       <c r="A118" s="16" t="n"/>
       <c r="B118" s="17" t="n"/>
       <c r="C118" s="17" t="n"/>
@@ -1838,7 +1769,7 @@
       <c r="G118" s="18" t="n"/>
       <c r="H118" s="17" t="n"/>
     </row>
-    <row r="119" ht="27" customHeight="1">
+    <row r="119" ht="19" customHeight="1">
       <c r="A119" s="16" t="n"/>
       <c r="B119" s="17" t="n"/>
       <c r="C119" s="17" t="n"/>
@@ -1848,7 +1779,7 @@
       <c r="G119" s="18" t="n"/>
       <c r="H119" s="17" t="n"/>
     </row>
-    <row r="120" ht="27" customHeight="1">
+    <row r="120" ht="19" customHeight="1">
       <c r="A120" s="16" t="n"/>
       <c r="B120" s="17" t="n"/>
       <c r="C120" s="17" t="n"/>
@@ -1858,7 +1789,7 @@
       <c r="G120" s="18" t="n"/>
       <c r="H120" s="17" t="n"/>
     </row>
-    <row r="121" ht="27" customHeight="1">
+    <row r="121" ht="19" customHeight="1">
       <c r="A121" s="16" t="n"/>
       <c r="B121" s="17" t="n"/>
       <c r="C121" s="17" t="n"/>
@@ -1868,7 +1799,7 @@
       <c r="G121" s="18" t="n"/>
       <c r="H121" s="17" t="n"/>
     </row>
-    <row r="122" ht="27" customHeight="1">
+    <row r="122" ht="19" customHeight="1">
       <c r="A122" s="16" t="n"/>
       <c r="B122" s="17" t="n"/>
       <c r="C122" s="17" t="n"/>
@@ -1878,7 +1809,7 @@
       <c r="G122" s="18" t="n"/>
       <c r="H122" s="17" t="n"/>
     </row>
-    <row r="123" ht="27" customHeight="1">
+    <row r="123" ht="19" customHeight="1">
       <c r="A123" s="16" t="n"/>
       <c r="B123" s="17" t="n"/>
       <c r="C123" s="17" t="n"/>
@@ -1888,7 +1819,7 @@
       <c r="G123" s="18" t="n"/>
       <c r="H123" s="17" t="n"/>
     </row>
-    <row r="124" ht="27" customHeight="1">
+    <row r="124" ht="19" customHeight="1">
       <c r="A124" s="16" t="n"/>
       <c r="B124" s="17" t="n"/>
       <c r="C124" s="17" t="n"/>
@@ -1898,7 +1829,7 @@
       <c r="G124" s="18" t="n"/>
       <c r="H124" s="17" t="n"/>
     </row>
-    <row r="125" ht="27" customHeight="1">
+    <row r="125" ht="19" customHeight="1">
       <c r="A125" s="16" t="n"/>
       <c r="B125" s="17" t="n"/>
       <c r="C125" s="17" t="n"/>
@@ -1908,7 +1839,7 @@
       <c r="G125" s="18" t="n"/>
       <c r="H125" s="17" t="n"/>
     </row>
-    <row r="126" ht="27" customHeight="1">
+    <row r="126" ht="19" customHeight="1">
       <c r="A126" s="16" t="n"/>
       <c r="B126" s="17" t="n"/>
       <c r="C126" s="17" t="n"/>
@@ -1918,7 +1849,7 @@
       <c r="G126" s="18" t="n"/>
       <c r="H126" s="17" t="n"/>
     </row>
-    <row r="127" ht="27" customHeight="1">
+    <row r="127" ht="19" customHeight="1">
       <c r="A127" s="16" t="n"/>
       <c r="B127" s="17" t="n"/>
       <c r="C127" s="17" t="n"/>
@@ -1928,7 +1859,7 @@
       <c r="G127" s="18" t="n"/>
       <c r="H127" s="17" t="n"/>
     </row>
-    <row r="128" ht="27" customHeight="1">
+    <row r="128" ht="19" customHeight="1">
       <c r="A128" s="16" t="n"/>
       <c r="B128" s="17" t="n"/>
       <c r="C128" s="17" t="n"/>
@@ -1938,7 +1869,7 @@
       <c r="G128" s="18" t="n"/>
       <c r="H128" s="17" t="n"/>
     </row>
-    <row r="129" ht="27" customHeight="1">
+    <row r="129" ht="19" customHeight="1">
       <c r="A129" s="16" t="n"/>
       <c r="B129" s="17" t="n"/>
       <c r="C129" s="17" t="n"/>
@@ -1948,7 +1879,7 @@
       <c r="G129" s="18" t="n"/>
       <c r="H129" s="17" t="n"/>
     </row>
-    <row r="130" ht="27" customHeight="1">
+    <row r="130" ht="19" customHeight="1">
       <c r="A130" s="16" t="n"/>
       <c r="B130" s="17" t="n"/>
       <c r="C130" s="17" t="n"/>
@@ -1958,7 +1889,7 @@
       <c r="G130" s="18" t="n"/>
       <c r="H130" s="17" t="n"/>
     </row>
-    <row r="131" ht="27" customHeight="1">
+    <row r="131" ht="19" customHeight="1">
       <c r="A131" s="16" t="n"/>
       <c r="B131" s="17" t="n"/>
       <c r="C131" s="17" t="n"/>
@@ -1968,47 +1899,77 @@
       <c r="G131" s="18" t="n"/>
       <c r="H131" s="17" t="n"/>
     </row>
-    <row r="132" ht="27" customHeight="1">
-      <c r="A132" s="16" t="n"/>
-      <c r="B132" s="17" t="n"/>
-      <c r="C132" s="17" t="n"/>
-      <c r="D132" s="16" t="n"/>
-      <c r="E132" s="16" t="n"/>
-      <c r="F132" s="18" t="n"/>
-      <c r="G132" s="18" t="n"/>
-      <c r="H132" s="17" t="n"/>
-    </row>
-    <row r="133" ht="27" customHeight="1">
-      <c r="A133" s="16" t="n"/>
-      <c r="B133" s="17" t="n"/>
-      <c r="C133" s="17" t="n"/>
-      <c r="D133" s="16" t="n"/>
-      <c r="E133" s="16" t="n"/>
-      <c r="F133" s="18" t="n"/>
-      <c r="G133" s="18" t="n"/>
-      <c r="H133" s="17" t="n"/>
-    </row>
-    <row r="134" ht="27" customHeight="1">
-      <c r="A134" s="16" t="n"/>
-      <c r="B134" s="17" t="n"/>
-      <c r="C134" s="17" t="n"/>
-      <c r="D134" s="16" t="n"/>
-      <c r="E134" s="16" t="n"/>
-      <c r="F134" s="18" t="n"/>
-      <c r="G134" s="18" t="n"/>
-      <c r="H134" s="17" t="n"/>
-    </row>
-    <row r="135" ht="27" customHeight="1">
-      <c r="A135" s="16" t="n"/>
-      <c r="B135" s="17" t="n"/>
-      <c r="C135" s="17" t="n"/>
-      <c r="D135" s="16" t="n"/>
-      <c r="E135" s="16" t="n"/>
-      <c r="F135" s="18" t="n"/>
-      <c r="G135" s="18" t="n"/>
-      <c r="H135" s="17" t="n"/>
-    </row>
-    <row r="136" ht="27" customHeight="1">
+    <row r="132" ht="18" customHeight="1">
+      <c r="A132" s="25" t="inlineStr">
+        <is>
+          <t>※工事内容明細には消費税が含まれておりません。</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="22" customHeight="1">
+      <c r="A133" s="26" t="n"/>
+      <c r="B133" s="26" t="n"/>
+      <c r="C133" s="26" t="n"/>
+      <c r="D133" s="26" t="n"/>
+      <c r="E133" s="26" t="n"/>
+      <c r="F133" s="27" t="inlineStr">
+        <is>
+          <t>合　計</t>
+        </is>
+      </c>
+      <c r="G133" s="28" t="n"/>
+      <c r="H133" s="26" t="n"/>
+    </row>
+    <row r="134" ht="22" customHeight="1">
+      <c r="A134" s="24" t="inlineStr">
+        <is>
+          <t>工 事 内 容 明 細</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="22" customHeight="1">
+      <c r="A135" s="15" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="B135" s="15" t="inlineStr">
+        <is>
+          <t>工事品目</t>
+        </is>
+      </c>
+      <c r="C135" s="15" t="inlineStr">
+        <is>
+          <t>仕様</t>
+        </is>
+      </c>
+      <c r="D135" s="15" t="inlineStr">
+        <is>
+          <t>数量</t>
+        </is>
+      </c>
+      <c r="E135" s="15" t="inlineStr">
+        <is>
+          <t>単位</t>
+        </is>
+      </c>
+      <c r="F135" s="15" t="inlineStr">
+        <is>
+          <t>単価</t>
+        </is>
+      </c>
+      <c r="G135" s="15" t="inlineStr">
+        <is>
+          <t>金額</t>
+        </is>
+      </c>
+      <c r="H135" s="15" t="inlineStr">
+        <is>
+          <t>備考</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" ht="19" customHeight="1">
       <c r="A136" s="16" t="n"/>
       <c r="B136" s="17" t="n"/>
       <c r="C136" s="17" t="n"/>
@@ -2018,7 +1979,7 @@
       <c r="G136" s="18" t="n"/>
       <c r="H136" s="17" t="n"/>
     </row>
-    <row r="137" ht="27" customHeight="1">
+    <row r="137" ht="19" customHeight="1">
       <c r="A137" s="16" t="n"/>
       <c r="B137" s="17" t="n"/>
       <c r="C137" s="17" t="n"/>
@@ -2028,7 +1989,7 @@
       <c r="G137" s="18" t="n"/>
       <c r="H137" s="17" t="n"/>
     </row>
-    <row r="138" ht="27" customHeight="1">
+    <row r="138" ht="19" customHeight="1">
       <c r="A138" s="16" t="n"/>
       <c r="B138" s="17" t="n"/>
       <c r="C138" s="17" t="n"/>
@@ -2038,7 +1999,7 @@
       <c r="G138" s="18" t="n"/>
       <c r="H138" s="17" t="n"/>
     </row>
-    <row r="139" ht="27" customHeight="1">
+    <row r="139" ht="19" customHeight="1">
       <c r="A139" s="16" t="n"/>
       <c r="B139" s="17" t="n"/>
       <c r="C139" s="17" t="n"/>
@@ -2048,7 +2009,7 @@
       <c r="G139" s="18" t="n"/>
       <c r="H139" s="17" t="n"/>
     </row>
-    <row r="140" ht="27" customHeight="1">
+    <row r="140" ht="19" customHeight="1">
       <c r="A140" s="16" t="n"/>
       <c r="B140" s="17" t="n"/>
       <c r="C140" s="17" t="n"/>
@@ -2058,7 +2019,7 @@
       <c r="G140" s="18" t="n"/>
       <c r="H140" s="17" t="n"/>
     </row>
-    <row r="141" ht="27" customHeight="1">
+    <row r="141" ht="19" customHeight="1">
       <c r="A141" s="16" t="n"/>
       <c r="B141" s="17" t="n"/>
       <c r="C141" s="17" t="n"/>
@@ -2068,7 +2029,7 @@
       <c r="G141" s="18" t="n"/>
       <c r="H141" s="17" t="n"/>
     </row>
-    <row r="142" ht="27" customHeight="1">
+    <row r="142" ht="19" customHeight="1">
       <c r="A142" s="16" t="n"/>
       <c r="B142" s="17" t="n"/>
       <c r="C142" s="17" t="n"/>
@@ -2078,7 +2039,7 @@
       <c r="G142" s="18" t="n"/>
       <c r="H142" s="17" t="n"/>
     </row>
-    <row r="143" ht="27" customHeight="1">
+    <row r="143" ht="19" customHeight="1">
       <c r="A143" s="16" t="n"/>
       <c r="B143" s="17" t="n"/>
       <c r="C143" s="17" t="n"/>
@@ -2088,7 +2049,7 @@
       <c r="G143" s="18" t="n"/>
       <c r="H143" s="17" t="n"/>
     </row>
-    <row r="144" ht="27" customHeight="1">
+    <row r="144" ht="19" customHeight="1">
       <c r="A144" s="16" t="n"/>
       <c r="B144" s="17" t="n"/>
       <c r="C144" s="17" t="n"/>
@@ -2098,7 +2059,7 @@
       <c r="G144" s="18" t="n"/>
       <c r="H144" s="17" t="n"/>
     </row>
-    <row r="145" ht="27" customHeight="1">
+    <row r="145" ht="19" customHeight="1">
       <c r="A145" s="16" t="n"/>
       <c r="B145" s="17" t="n"/>
       <c r="C145" s="17" t="n"/>
@@ -2108,7 +2069,7 @@
       <c r="G145" s="18" t="n"/>
       <c r="H145" s="17" t="n"/>
     </row>
-    <row r="146" ht="27" customHeight="1">
+    <row r="146" ht="19" customHeight="1">
       <c r="A146" s="16" t="n"/>
       <c r="B146" s="17" t="n"/>
       <c r="C146" s="17" t="n"/>
@@ -2118,7 +2079,7 @@
       <c r="G146" s="18" t="n"/>
       <c r="H146" s="17" t="n"/>
     </row>
-    <row r="147" ht="27" customHeight="1">
+    <row r="147" ht="19" customHeight="1">
       <c r="A147" s="16" t="n"/>
       <c r="B147" s="17" t="n"/>
       <c r="C147" s="17" t="n"/>
@@ -2128,7 +2089,7 @@
       <c r="G147" s="18" t="n"/>
       <c r="H147" s="17" t="n"/>
     </row>
-    <row r="148" ht="27" customHeight="1">
+    <row r="148" ht="19" customHeight="1">
       <c r="A148" s="16" t="n"/>
       <c r="B148" s="17" t="n"/>
       <c r="C148" s="17" t="n"/>
@@ -2138,7 +2099,7 @@
       <c r="G148" s="18" t="n"/>
       <c r="H148" s="17" t="n"/>
     </row>
-    <row r="149" ht="27" customHeight="1">
+    <row r="149" ht="19" customHeight="1">
       <c r="A149" s="16" t="n"/>
       <c r="B149" s="17" t="n"/>
       <c r="C149" s="17" t="n"/>
@@ -2148,7 +2109,7 @@
       <c r="G149" s="18" t="n"/>
       <c r="H149" s="17" t="n"/>
     </row>
-    <row r="150" ht="27" customHeight="1">
+    <row r="150" ht="19" customHeight="1">
       <c r="A150" s="16" t="n"/>
       <c r="B150" s="17" t="n"/>
       <c r="C150" s="17" t="n"/>
@@ -2158,7 +2119,7 @@
       <c r="G150" s="18" t="n"/>
       <c r="H150" s="17" t="n"/>
     </row>
-    <row r="151" ht="27" customHeight="1">
+    <row r="151" ht="19" customHeight="1">
       <c r="A151" s="16" t="n"/>
       <c r="B151" s="17" t="n"/>
       <c r="C151" s="17" t="n"/>
@@ -2168,7 +2129,7 @@
       <c r="G151" s="18" t="n"/>
       <c r="H151" s="17" t="n"/>
     </row>
-    <row r="152" ht="27" customHeight="1">
+    <row r="152" ht="19" customHeight="1">
       <c r="A152" s="16" t="n"/>
       <c r="B152" s="17" t="n"/>
       <c r="C152" s="17" t="n"/>
@@ -2178,7 +2139,7 @@
       <c r="G152" s="18" t="n"/>
       <c r="H152" s="17" t="n"/>
     </row>
-    <row r="153" ht="27" customHeight="1">
+    <row r="153" ht="19" customHeight="1">
       <c r="A153" s="16" t="n"/>
       <c r="B153" s="17" t="n"/>
       <c r="C153" s="17" t="n"/>
@@ -2188,7 +2149,7 @@
       <c r="G153" s="18" t="n"/>
       <c r="H153" s="17" t="n"/>
     </row>
-    <row r="154" ht="27" customHeight="1">
+    <row r="154" ht="19" customHeight="1">
       <c r="A154" s="16" t="n"/>
       <c r="B154" s="17" t="n"/>
       <c r="C154" s="17" t="n"/>
@@ -2198,7 +2159,7 @@
       <c r="G154" s="18" t="n"/>
       <c r="H154" s="17" t="n"/>
     </row>
-    <row r="155" ht="27" customHeight="1">
+    <row r="155" ht="19" customHeight="1">
       <c r="A155" s="16" t="n"/>
       <c r="B155" s="17" t="n"/>
       <c r="C155" s="17" t="n"/>
@@ -2208,47 +2169,77 @@
       <c r="G155" s="18" t="n"/>
       <c r="H155" s="17" t="n"/>
     </row>
-    <row r="156" ht="27" customHeight="1">
-      <c r="A156" s="16" t="n"/>
-      <c r="B156" s="17" t="n"/>
-      <c r="C156" s="17" t="n"/>
-      <c r="D156" s="16" t="n"/>
-      <c r="E156" s="16" t="n"/>
-      <c r="F156" s="18" t="n"/>
-      <c r="G156" s="18" t="n"/>
-      <c r="H156" s="17" t="n"/>
-    </row>
-    <row r="157" ht="27" customHeight="1">
-      <c r="A157" s="16" t="n"/>
-      <c r="B157" s="17" t="n"/>
-      <c r="C157" s="17" t="n"/>
-      <c r="D157" s="16" t="n"/>
-      <c r="E157" s="16" t="n"/>
-      <c r="F157" s="18" t="n"/>
-      <c r="G157" s="18" t="n"/>
-      <c r="H157" s="17" t="n"/>
-    </row>
-    <row r="158" ht="27" customHeight="1">
-      <c r="A158" s="16" t="n"/>
-      <c r="B158" s="17" t="n"/>
-      <c r="C158" s="17" t="n"/>
-      <c r="D158" s="16" t="n"/>
-      <c r="E158" s="16" t="n"/>
-      <c r="F158" s="18" t="n"/>
-      <c r="G158" s="18" t="n"/>
-      <c r="H158" s="17" t="n"/>
-    </row>
-    <row r="159" ht="27" customHeight="1">
-      <c r="A159" s="16" t="n"/>
-      <c r="B159" s="17" t="n"/>
-      <c r="C159" s="17" t="n"/>
-      <c r="D159" s="16" t="n"/>
-      <c r="E159" s="16" t="n"/>
-      <c r="F159" s="18" t="n"/>
-      <c r="G159" s="18" t="n"/>
-      <c r="H159" s="17" t="n"/>
-    </row>
-    <row r="160" ht="27" customHeight="1">
+    <row r="156" ht="18" customHeight="1">
+      <c r="A156" s="25" t="inlineStr">
+        <is>
+          <t>※工事内容明細には消費税が含まれておりません。</t>
+        </is>
+      </c>
+    </row>
+    <row r="157" ht="22" customHeight="1">
+      <c r="A157" s="26" t="n"/>
+      <c r="B157" s="26" t="n"/>
+      <c r="C157" s="26" t="n"/>
+      <c r="D157" s="26" t="n"/>
+      <c r="E157" s="26" t="n"/>
+      <c r="F157" s="27" t="inlineStr">
+        <is>
+          <t>合　計</t>
+        </is>
+      </c>
+      <c r="G157" s="28" t="n"/>
+      <c r="H157" s="26" t="n"/>
+    </row>
+    <row r="158" ht="22" customHeight="1">
+      <c r="A158" s="24" t="inlineStr">
+        <is>
+          <t>工 事 内 容 明 細</t>
+        </is>
+      </c>
+    </row>
+    <row r="159" ht="22" customHeight="1">
+      <c r="A159" s="15" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="B159" s="15" t="inlineStr">
+        <is>
+          <t>工事品目</t>
+        </is>
+      </c>
+      <c r="C159" s="15" t="inlineStr">
+        <is>
+          <t>仕様</t>
+        </is>
+      </c>
+      <c r="D159" s="15" t="inlineStr">
+        <is>
+          <t>数量</t>
+        </is>
+      </c>
+      <c r="E159" s="15" t="inlineStr">
+        <is>
+          <t>単位</t>
+        </is>
+      </c>
+      <c r="F159" s="15" t="inlineStr">
+        <is>
+          <t>単価</t>
+        </is>
+      </c>
+      <c r="G159" s="15" t="inlineStr">
+        <is>
+          <t>金額</t>
+        </is>
+      </c>
+      <c r="H159" s="15" t="inlineStr">
+        <is>
+          <t>備考</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" ht="19" customHeight="1">
       <c r="A160" s="16" t="n"/>
       <c r="B160" s="17" t="n"/>
       <c r="C160" s="17" t="n"/>
@@ -2258,7 +2249,7 @@
       <c r="G160" s="18" t="n"/>
       <c r="H160" s="17" t="n"/>
     </row>
-    <row r="161" ht="27" customHeight="1">
+    <row r="161" ht="19" customHeight="1">
       <c r="A161" s="16" t="n"/>
       <c r="B161" s="17" t="n"/>
       <c r="C161" s="17" t="n"/>
@@ -2268,7 +2259,7 @@
       <c r="G161" s="18" t="n"/>
       <c r="H161" s="17" t="n"/>
     </row>
-    <row r="162" ht="27" customHeight="1">
+    <row r="162" ht="19" customHeight="1">
       <c r="A162" s="16" t="n"/>
       <c r="B162" s="17" t="n"/>
       <c r="C162" s="17" t="n"/>
@@ -2278,7 +2269,7 @@
       <c r="G162" s="18" t="n"/>
       <c r="H162" s="17" t="n"/>
     </row>
-    <row r="163" ht="27" customHeight="1">
+    <row r="163" ht="19" customHeight="1">
       <c r="A163" s="16" t="n"/>
       <c r="B163" s="17" t="n"/>
       <c r="C163" s="17" t="n"/>
@@ -2288,7 +2279,7 @@
       <c r="G163" s="18" t="n"/>
       <c r="H163" s="17" t="n"/>
     </row>
-    <row r="164" ht="27" customHeight="1">
+    <row r="164" ht="19" customHeight="1">
       <c r="A164" s="16" t="n"/>
       <c r="B164" s="17" t="n"/>
       <c r="C164" s="17" t="n"/>
@@ -2298,7 +2289,7 @@
       <c r="G164" s="18" t="n"/>
       <c r="H164" s="17" t="n"/>
     </row>
-    <row r="165" ht="27" customHeight="1">
+    <row r="165" ht="19" customHeight="1">
       <c r="A165" s="16" t="n"/>
       <c r="B165" s="17" t="n"/>
       <c r="C165" s="17" t="n"/>
@@ -2308,7 +2299,7 @@
       <c r="G165" s="18" t="n"/>
       <c r="H165" s="17" t="n"/>
     </row>
-    <row r="166" ht="27" customHeight="1">
+    <row r="166" ht="19" customHeight="1">
       <c r="A166" s="16" t="n"/>
       <c r="B166" s="17" t="n"/>
       <c r="C166" s="17" t="n"/>
@@ -2318,7 +2309,7 @@
       <c r="G166" s="18" t="n"/>
       <c r="H166" s="17" t="n"/>
     </row>
-    <row r="167" ht="27" customHeight="1">
+    <row r="167" ht="19" customHeight="1">
       <c r="A167" s="16" t="n"/>
       <c r="B167" s="17" t="n"/>
       <c r="C167" s="17" t="n"/>
@@ -2328,7 +2319,7 @@
       <c r="G167" s="18" t="n"/>
       <c r="H167" s="17" t="n"/>
     </row>
-    <row r="168" ht="27" customHeight="1">
+    <row r="168" ht="19" customHeight="1">
       <c r="A168" s="16" t="n"/>
       <c r="B168" s="17" t="n"/>
       <c r="C168" s="17" t="n"/>
@@ -2338,7 +2329,7 @@
       <c r="G168" s="18" t="n"/>
       <c r="H168" s="17" t="n"/>
     </row>
-    <row r="169" ht="27" customHeight="1">
+    <row r="169" ht="19" customHeight="1">
       <c r="A169" s="16" t="n"/>
       <c r="B169" s="17" t="n"/>
       <c r="C169" s="17" t="n"/>
@@ -2348,7 +2339,7 @@
       <c r="G169" s="18" t="n"/>
       <c r="H169" s="17" t="n"/>
     </row>
-    <row r="170" ht="27" customHeight="1">
+    <row r="170" ht="19" customHeight="1">
       <c r="A170" s="16" t="n"/>
       <c r="B170" s="17" t="n"/>
       <c r="C170" s="17" t="n"/>
@@ -2358,112 +2349,990 @@
       <c r="G170" s="18" t="n"/>
       <c r="H170" s="17" t="n"/>
     </row>
-    <row r="171" ht="27" customHeight="1">
-      <c r="A171" s="19" t="n"/>
-      <c r="B171" s="20" t="n"/>
-      <c r="C171" s="20" t="n"/>
-      <c r="D171" s="19" t="n"/>
-      <c r="E171" s="19" t="n"/>
-      <c r="F171" s="21" t="n"/>
-      <c r="G171" s="21" t="n"/>
-      <c r="H171" s="20" t="n"/>
-    </row>
-    <row r="172" ht="6" customHeight="1"/>
-    <row r="173" ht="17" customHeight="1">
-      <c r="E173" s="22" t="inlineStr">
-        <is>
-          <t>小　　計</t>
-        </is>
-      </c>
-      <c r="G173" s="23" t="n"/>
-    </row>
-    <row r="174" ht="17" customHeight="1">
-      <c r="E174" s="22" t="inlineStr">
-        <is>
-          <t>値 引 き</t>
-        </is>
-      </c>
-      <c r="G174" s="23" t="n"/>
-    </row>
-    <row r="175" ht="17" customHeight="1">
-      <c r="E175" s="22" t="inlineStr">
-        <is>
-          <t>税抜合計</t>
-        </is>
-      </c>
-      <c r="G175" s="23" t="n"/>
-    </row>
-    <row r="176" ht="17" customHeight="1">
-      <c r="E176" s="22" t="inlineStr">
-        <is>
-          <t>消 費 税</t>
-        </is>
-      </c>
-      <c r="G176" s="23" t="n"/>
-    </row>
-    <row r="177" ht="23" customHeight="1">
-      <c r="E177" s="24" t="inlineStr">
-        <is>
-          <t>税込合計</t>
-        </is>
-      </c>
-      <c r="G177" s="25" t="n"/>
-    </row>
-    <row r="178" ht="6" customHeight="1"/>
-    <row r="179">
-      <c r="A179" s="5" t="inlineStr">
+    <row r="171" ht="19" customHeight="1">
+      <c r="A171" s="16" t="n"/>
+      <c r="B171" s="17" t="n"/>
+      <c r="C171" s="17" t="n"/>
+      <c r="D171" s="16" t="n"/>
+      <c r="E171" s="16" t="n"/>
+      <c r="F171" s="18" t="n"/>
+      <c r="G171" s="18" t="n"/>
+      <c r="H171" s="17" t="n"/>
+    </row>
+    <row r="172" ht="19" customHeight="1">
+      <c r="A172" s="16" t="n"/>
+      <c r="B172" s="17" t="n"/>
+      <c r="C172" s="17" t="n"/>
+      <c r="D172" s="16" t="n"/>
+      <c r="E172" s="16" t="n"/>
+      <c r="F172" s="18" t="n"/>
+      <c r="G172" s="18" t="n"/>
+      <c r="H172" s="17" t="n"/>
+    </row>
+    <row r="173" ht="19" customHeight="1">
+      <c r="A173" s="16" t="n"/>
+      <c r="B173" s="17" t="n"/>
+      <c r="C173" s="17" t="n"/>
+      <c r="D173" s="16" t="n"/>
+      <c r="E173" s="16" t="n"/>
+      <c r="F173" s="18" t="n"/>
+      <c r="G173" s="18" t="n"/>
+      <c r="H173" s="17" t="n"/>
+    </row>
+    <row r="174" ht="19" customHeight="1">
+      <c r="A174" s="16" t="n"/>
+      <c r="B174" s="17" t="n"/>
+      <c r="C174" s="17" t="n"/>
+      <c r="D174" s="16" t="n"/>
+      <c r="E174" s="16" t="n"/>
+      <c r="F174" s="18" t="n"/>
+      <c r="G174" s="18" t="n"/>
+      <c r="H174" s="17" t="n"/>
+    </row>
+    <row r="175" ht="19" customHeight="1">
+      <c r="A175" s="16" t="n"/>
+      <c r="B175" s="17" t="n"/>
+      <c r="C175" s="17" t="n"/>
+      <c r="D175" s="16" t="n"/>
+      <c r="E175" s="16" t="n"/>
+      <c r="F175" s="18" t="n"/>
+      <c r="G175" s="18" t="n"/>
+      <c r="H175" s="17" t="n"/>
+    </row>
+    <row r="176" ht="19" customHeight="1">
+      <c r="A176" s="16" t="n"/>
+      <c r="B176" s="17" t="n"/>
+      <c r="C176" s="17" t="n"/>
+      <c r="D176" s="16" t="n"/>
+      <c r="E176" s="16" t="n"/>
+      <c r="F176" s="18" t="n"/>
+      <c r="G176" s="18" t="n"/>
+      <c r="H176" s="17" t="n"/>
+    </row>
+    <row r="177" ht="19" customHeight="1">
+      <c r="A177" s="16" t="n"/>
+      <c r="B177" s="17" t="n"/>
+      <c r="C177" s="17" t="n"/>
+      <c r="D177" s="16" t="n"/>
+      <c r="E177" s="16" t="n"/>
+      <c r="F177" s="18" t="n"/>
+      <c r="G177" s="18" t="n"/>
+      <c r="H177" s="17" t="n"/>
+    </row>
+    <row r="178" ht="19" customHeight="1">
+      <c r="A178" s="16" t="n"/>
+      <c r="B178" s="17" t="n"/>
+      <c r="C178" s="17" t="n"/>
+      <c r="D178" s="16" t="n"/>
+      <c r="E178" s="16" t="n"/>
+      <c r="F178" s="18" t="n"/>
+      <c r="G178" s="18" t="n"/>
+      <c r="H178" s="17" t="n"/>
+    </row>
+    <row r="179" ht="19" customHeight="1">
+      <c r="A179" s="16" t="n"/>
+      <c r="B179" s="17" t="n"/>
+      <c r="C179" s="17" t="n"/>
+      <c r="D179" s="16" t="n"/>
+      <c r="E179" s="16" t="n"/>
+      <c r="F179" s="18" t="n"/>
+      <c r="G179" s="18" t="n"/>
+      <c r="H179" s="17" t="n"/>
+    </row>
+    <row r="180" ht="18" customHeight="1">
+      <c r="A180" s="25" t="inlineStr">
+        <is>
+          <t>※工事内容明細には消費税が含まれておりません。</t>
+        </is>
+      </c>
+    </row>
+    <row r="181" ht="22" customHeight="1">
+      <c r="A181" s="26" t="n"/>
+      <c r="B181" s="26" t="n"/>
+      <c r="C181" s="26" t="n"/>
+      <c r="D181" s="26" t="n"/>
+      <c r="E181" s="26" t="n"/>
+      <c r="F181" s="27" t="inlineStr">
+        <is>
+          <t>合　計</t>
+        </is>
+      </c>
+      <c r="G181" s="28" t="n"/>
+      <c r="H181" s="26" t="n"/>
+    </row>
+    <row r="182" ht="22" customHeight="1">
+      <c r="A182" s="24" t="inlineStr">
+        <is>
+          <t>工 事 内 容 明 細</t>
+        </is>
+      </c>
+    </row>
+    <row r="183" ht="22" customHeight="1">
+      <c r="A183" s="15" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="B183" s="15" t="inlineStr">
+        <is>
+          <t>工事品目</t>
+        </is>
+      </c>
+      <c r="C183" s="15" t="inlineStr">
+        <is>
+          <t>仕様</t>
+        </is>
+      </c>
+      <c r="D183" s="15" t="inlineStr">
+        <is>
+          <t>数量</t>
+        </is>
+      </c>
+      <c r="E183" s="15" t="inlineStr">
+        <is>
+          <t>単位</t>
+        </is>
+      </c>
+      <c r="F183" s="15" t="inlineStr">
+        <is>
+          <t>単価</t>
+        </is>
+      </c>
+      <c r="G183" s="15" t="inlineStr">
+        <is>
+          <t>金額</t>
+        </is>
+      </c>
+      <c r="H183" s="15" t="inlineStr">
         <is>
           <t>備考</t>
         </is>
       </c>
-      <c r="B179" s="26" t="n"/>
-    </row>
-    <row r="180"/>
-    <row r="181" ht="6" customHeight="1"/>
-    <row r="182" ht="12" customHeight="1">
-      <c r="A182" s="27" t="inlineStr">
-        <is>
-          <t>※本見積書の有効期限を過ぎた場合は、再度お見積りいたします。</t>
-        </is>
-      </c>
+    </row>
+    <row r="184" ht="19" customHeight="1">
+      <c r="A184" s="16" t="n"/>
+      <c r="B184" s="17" t="n"/>
+      <c r="C184" s="17" t="n"/>
+      <c r="D184" s="16" t="n"/>
+      <c r="E184" s="16" t="n"/>
+      <c r="F184" s="18" t="n"/>
+      <c r="G184" s="18" t="n"/>
+      <c r="H184" s="17" t="n"/>
+    </row>
+    <row r="185" ht="19" customHeight="1">
+      <c r="A185" s="16" t="n"/>
+      <c r="B185" s="17" t="n"/>
+      <c r="C185" s="17" t="n"/>
+      <c r="D185" s="16" t="n"/>
+      <c r="E185" s="16" t="n"/>
+      <c r="F185" s="18" t="n"/>
+      <c r="G185" s="18" t="n"/>
+      <c r="H185" s="17" t="n"/>
+    </row>
+    <row r="186" ht="19" customHeight="1">
+      <c r="A186" s="16" t="n"/>
+      <c r="B186" s="17" t="n"/>
+      <c r="C186" s="17" t="n"/>
+      <c r="D186" s="16" t="n"/>
+      <c r="E186" s="16" t="n"/>
+      <c r="F186" s="18" t="n"/>
+      <c r="G186" s="18" t="n"/>
+      <c r="H186" s="17" t="n"/>
+    </row>
+    <row r="187" ht="19" customHeight="1">
+      <c r="A187" s="16" t="n"/>
+      <c r="B187" s="17" t="n"/>
+      <c r="C187" s="17" t="n"/>
+      <c r="D187" s="16" t="n"/>
+      <c r="E187" s="16" t="n"/>
+      <c r="F187" s="18" t="n"/>
+      <c r="G187" s="18" t="n"/>
+      <c r="H187" s="17" t="n"/>
+    </row>
+    <row r="188" ht="19" customHeight="1">
+      <c r="A188" s="16" t="n"/>
+      <c r="B188" s="17" t="n"/>
+      <c r="C188" s="17" t="n"/>
+      <c r="D188" s="16" t="n"/>
+      <c r="E188" s="16" t="n"/>
+      <c r="F188" s="18" t="n"/>
+      <c r="G188" s="18" t="n"/>
+      <c r="H188" s="17" t="n"/>
+    </row>
+    <row r="189" ht="19" customHeight="1">
+      <c r="A189" s="16" t="n"/>
+      <c r="B189" s="17" t="n"/>
+      <c r="C189" s="17" t="n"/>
+      <c r="D189" s="16" t="n"/>
+      <c r="E189" s="16" t="n"/>
+      <c r="F189" s="18" t="n"/>
+      <c r="G189" s="18" t="n"/>
+      <c r="H189" s="17" t="n"/>
+    </row>
+    <row r="190" ht="19" customHeight="1">
+      <c r="A190" s="16" t="n"/>
+      <c r="B190" s="17" t="n"/>
+      <c r="C190" s="17" t="n"/>
+      <c r="D190" s="16" t="n"/>
+      <c r="E190" s="16" t="n"/>
+      <c r="F190" s="18" t="n"/>
+      <c r="G190" s="18" t="n"/>
+      <c r="H190" s="17" t="n"/>
+    </row>
+    <row r="191" ht="19" customHeight="1">
+      <c r="A191" s="16" t="n"/>
+      <c r="B191" s="17" t="n"/>
+      <c r="C191" s="17" t="n"/>
+      <c r="D191" s="16" t="n"/>
+      <c r="E191" s="16" t="n"/>
+      <c r="F191" s="18" t="n"/>
+      <c r="G191" s="18" t="n"/>
+      <c r="H191" s="17" t="n"/>
+    </row>
+    <row r="192" ht="19" customHeight="1">
+      <c r="A192" s="16" t="n"/>
+      <c r="B192" s="17" t="n"/>
+      <c r="C192" s="17" t="n"/>
+      <c r="D192" s="16" t="n"/>
+      <c r="E192" s="16" t="n"/>
+      <c r="F192" s="18" t="n"/>
+      <c r="G192" s="18" t="n"/>
+      <c r="H192" s="17" t="n"/>
+    </row>
+    <row r="193" ht="19" customHeight="1">
+      <c r="A193" s="16" t="n"/>
+      <c r="B193" s="17" t="n"/>
+      <c r="C193" s="17" t="n"/>
+      <c r="D193" s="16" t="n"/>
+      <c r="E193" s="16" t="n"/>
+      <c r="F193" s="18" t="n"/>
+      <c r="G193" s="18" t="n"/>
+      <c r="H193" s="17" t="n"/>
+    </row>
+    <row r="194" ht="19" customHeight="1">
+      <c r="A194" s="16" t="n"/>
+      <c r="B194" s="17" t="n"/>
+      <c r="C194" s="17" t="n"/>
+      <c r="D194" s="16" t="n"/>
+      <c r="E194" s="16" t="n"/>
+      <c r="F194" s="18" t="n"/>
+      <c r="G194" s="18" t="n"/>
+      <c r="H194" s="17" t="n"/>
+    </row>
+    <row r="195" ht="19" customHeight="1">
+      <c r="A195" s="16" t="n"/>
+      <c r="B195" s="17" t="n"/>
+      <c r="C195" s="17" t="n"/>
+      <c r="D195" s="16" t="n"/>
+      <c r="E195" s="16" t="n"/>
+      <c r="F195" s="18" t="n"/>
+      <c r="G195" s="18" t="n"/>
+      <c r="H195" s="17" t="n"/>
+    </row>
+    <row r="196" ht="19" customHeight="1">
+      <c r="A196" s="16" t="n"/>
+      <c r="B196" s="17" t="n"/>
+      <c r="C196" s="17" t="n"/>
+      <c r="D196" s="16" t="n"/>
+      <c r="E196" s="16" t="n"/>
+      <c r="F196" s="18" t="n"/>
+      <c r="G196" s="18" t="n"/>
+      <c r="H196" s="17" t="n"/>
+    </row>
+    <row r="197" ht="19" customHeight="1">
+      <c r="A197" s="16" t="n"/>
+      <c r="B197" s="17" t="n"/>
+      <c r="C197" s="17" t="n"/>
+      <c r="D197" s="16" t="n"/>
+      <c r="E197" s="16" t="n"/>
+      <c r="F197" s="18" t="n"/>
+      <c r="G197" s="18" t="n"/>
+      <c r="H197" s="17" t="n"/>
+    </row>
+    <row r="198" ht="19" customHeight="1">
+      <c r="A198" s="16" t="n"/>
+      <c r="B198" s="17" t="n"/>
+      <c r="C198" s="17" t="n"/>
+      <c r="D198" s="16" t="n"/>
+      <c r="E198" s="16" t="n"/>
+      <c r="F198" s="18" t="n"/>
+      <c r="G198" s="18" t="n"/>
+      <c r="H198" s="17" t="n"/>
+    </row>
+    <row r="199" ht="19" customHeight="1">
+      <c r="A199" s="16" t="n"/>
+      <c r="B199" s="17" t="n"/>
+      <c r="C199" s="17" t="n"/>
+      <c r="D199" s="16" t="n"/>
+      <c r="E199" s="16" t="n"/>
+      <c r="F199" s="18" t="n"/>
+      <c r="G199" s="18" t="n"/>
+      <c r="H199" s="17" t="n"/>
+    </row>
+    <row r="200" ht="19" customHeight="1">
+      <c r="A200" s="16" t="n"/>
+      <c r="B200" s="17" t="n"/>
+      <c r="C200" s="17" t="n"/>
+      <c r="D200" s="16" t="n"/>
+      <c r="E200" s="16" t="n"/>
+      <c r="F200" s="18" t="n"/>
+      <c r="G200" s="18" t="n"/>
+      <c r="H200" s="17" t="n"/>
+    </row>
+    <row r="201" ht="19" customHeight="1">
+      <c r="A201" s="16" t="n"/>
+      <c r="B201" s="17" t="n"/>
+      <c r="C201" s="17" t="n"/>
+      <c r="D201" s="16" t="n"/>
+      <c r="E201" s="16" t="n"/>
+      <c r="F201" s="18" t="n"/>
+      <c r="G201" s="18" t="n"/>
+      <c r="H201" s="17" t="n"/>
+    </row>
+    <row r="202" ht="19" customHeight="1">
+      <c r="A202" s="16" t="n"/>
+      <c r="B202" s="17" t="n"/>
+      <c r="C202" s="17" t="n"/>
+      <c r="D202" s="16" t="n"/>
+      <c r="E202" s="16" t="n"/>
+      <c r="F202" s="18" t="n"/>
+      <c r="G202" s="18" t="n"/>
+      <c r="H202" s="17" t="n"/>
+    </row>
+    <row r="203" ht="19" customHeight="1">
+      <c r="A203" s="16" t="n"/>
+      <c r="B203" s="17" t="n"/>
+      <c r="C203" s="17" t="n"/>
+      <c r="D203" s="16" t="n"/>
+      <c r="E203" s="16" t="n"/>
+      <c r="F203" s="18" t="n"/>
+      <c r="G203" s="18" t="n"/>
+      <c r="H203" s="17" t="n"/>
+    </row>
+    <row r="204" ht="18" customHeight="1">
+      <c r="A204" s="25" t="inlineStr">
+        <is>
+          <t>※工事内容明細には消費税が含まれておりません。</t>
+        </is>
+      </c>
+    </row>
+    <row r="205" ht="22" customHeight="1">
+      <c r="A205" s="26" t="n"/>
+      <c r="B205" s="26" t="n"/>
+      <c r="C205" s="26" t="n"/>
+      <c r="D205" s="26" t="n"/>
+      <c r="E205" s="26" t="n"/>
+      <c r="F205" s="27" t="inlineStr">
+        <is>
+          <t>合　計</t>
+        </is>
+      </c>
+      <c r="G205" s="28" t="n"/>
+      <c r="H205" s="26" t="n"/>
+    </row>
+    <row r="206" ht="22" customHeight="1">
+      <c r="A206" s="24" t="inlineStr">
+        <is>
+          <t>工 事 内 容 明 細</t>
+        </is>
+      </c>
+    </row>
+    <row r="207" ht="22" customHeight="1">
+      <c r="A207" s="15" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="B207" s="15" t="inlineStr">
+        <is>
+          <t>工事品目</t>
+        </is>
+      </c>
+      <c r="C207" s="15" t="inlineStr">
+        <is>
+          <t>仕様</t>
+        </is>
+      </c>
+      <c r="D207" s="15" t="inlineStr">
+        <is>
+          <t>数量</t>
+        </is>
+      </c>
+      <c r="E207" s="15" t="inlineStr">
+        <is>
+          <t>単位</t>
+        </is>
+      </c>
+      <c r="F207" s="15" t="inlineStr">
+        <is>
+          <t>単価</t>
+        </is>
+      </c>
+      <c r="G207" s="15" t="inlineStr">
+        <is>
+          <t>金額</t>
+        </is>
+      </c>
+      <c r="H207" s="15" t="inlineStr">
+        <is>
+          <t>備考</t>
+        </is>
+      </c>
+    </row>
+    <row r="208" ht="19" customHeight="1">
+      <c r="A208" s="16" t="n"/>
+      <c r="B208" s="17" t="n"/>
+      <c r="C208" s="17" t="n"/>
+      <c r="D208" s="16" t="n"/>
+      <c r="E208" s="16" t="n"/>
+      <c r="F208" s="18" t="n"/>
+      <c r="G208" s="18" t="n"/>
+      <c r="H208" s="17" t="n"/>
+    </row>
+    <row r="209" ht="19" customHeight="1">
+      <c r="A209" s="16" t="n"/>
+      <c r="B209" s="17" t="n"/>
+      <c r="C209" s="17" t="n"/>
+      <c r="D209" s="16" t="n"/>
+      <c r="E209" s="16" t="n"/>
+      <c r="F209" s="18" t="n"/>
+      <c r="G209" s="18" t="n"/>
+      <c r="H209" s="17" t="n"/>
+    </row>
+    <row r="210" ht="19" customHeight="1">
+      <c r="A210" s="16" t="n"/>
+      <c r="B210" s="17" t="n"/>
+      <c r="C210" s="17" t="n"/>
+      <c r="D210" s="16" t="n"/>
+      <c r="E210" s="16" t="n"/>
+      <c r="F210" s="18" t="n"/>
+      <c r="G210" s="18" t="n"/>
+      <c r="H210" s="17" t="n"/>
+    </row>
+    <row r="211" ht="19" customHeight="1">
+      <c r="A211" s="16" t="n"/>
+      <c r="B211" s="17" t="n"/>
+      <c r="C211" s="17" t="n"/>
+      <c r="D211" s="16" t="n"/>
+      <c r="E211" s="16" t="n"/>
+      <c r="F211" s="18" t="n"/>
+      <c r="G211" s="18" t="n"/>
+      <c r="H211" s="17" t="n"/>
+    </row>
+    <row r="212" ht="19" customHeight="1">
+      <c r="A212" s="16" t="n"/>
+      <c r="B212" s="17" t="n"/>
+      <c r="C212" s="17" t="n"/>
+      <c r="D212" s="16" t="n"/>
+      <c r="E212" s="16" t="n"/>
+      <c r="F212" s="18" t="n"/>
+      <c r="G212" s="18" t="n"/>
+      <c r="H212" s="17" t="n"/>
+    </row>
+    <row r="213" ht="19" customHeight="1">
+      <c r="A213" s="16" t="n"/>
+      <c r="B213" s="17" t="n"/>
+      <c r="C213" s="17" t="n"/>
+      <c r="D213" s="16" t="n"/>
+      <c r="E213" s="16" t="n"/>
+      <c r="F213" s="18" t="n"/>
+      <c r="G213" s="18" t="n"/>
+      <c r="H213" s="17" t="n"/>
+    </row>
+    <row r="214" ht="19" customHeight="1">
+      <c r="A214" s="16" t="n"/>
+      <c r="B214" s="17" t="n"/>
+      <c r="C214" s="17" t="n"/>
+      <c r="D214" s="16" t="n"/>
+      <c r="E214" s="16" t="n"/>
+      <c r="F214" s="18" t="n"/>
+      <c r="G214" s="18" t="n"/>
+      <c r="H214" s="17" t="n"/>
+    </row>
+    <row r="215" ht="19" customHeight="1">
+      <c r="A215" s="16" t="n"/>
+      <c r="B215" s="17" t="n"/>
+      <c r="C215" s="17" t="n"/>
+      <c r="D215" s="16" t="n"/>
+      <c r="E215" s="16" t="n"/>
+      <c r="F215" s="18" t="n"/>
+      <c r="G215" s="18" t="n"/>
+      <c r="H215" s="17" t="n"/>
+    </row>
+    <row r="216" ht="19" customHeight="1">
+      <c r="A216" s="16" t="n"/>
+      <c r="B216" s="17" t="n"/>
+      <c r="C216" s="17" t="n"/>
+      <c r="D216" s="16" t="n"/>
+      <c r="E216" s="16" t="n"/>
+      <c r="F216" s="18" t="n"/>
+      <c r="G216" s="18" t="n"/>
+      <c r="H216" s="17" t="n"/>
+    </row>
+    <row r="217" ht="19" customHeight="1">
+      <c r="A217" s="16" t="n"/>
+      <c r="B217" s="17" t="n"/>
+      <c r="C217" s="17" t="n"/>
+      <c r="D217" s="16" t="n"/>
+      <c r="E217" s="16" t="n"/>
+      <c r="F217" s="18" t="n"/>
+      <c r="G217" s="18" t="n"/>
+      <c r="H217" s="17" t="n"/>
+    </row>
+    <row r="218" ht="19" customHeight="1">
+      <c r="A218" s="16" t="n"/>
+      <c r="B218" s="17" t="n"/>
+      <c r="C218" s="17" t="n"/>
+      <c r="D218" s="16" t="n"/>
+      <c r="E218" s="16" t="n"/>
+      <c r="F218" s="18" t="n"/>
+      <c r="G218" s="18" t="n"/>
+      <c r="H218" s="17" t="n"/>
+    </row>
+    <row r="219" ht="19" customHeight="1">
+      <c r="A219" s="16" t="n"/>
+      <c r="B219" s="17" t="n"/>
+      <c r="C219" s="17" t="n"/>
+      <c r="D219" s="16" t="n"/>
+      <c r="E219" s="16" t="n"/>
+      <c r="F219" s="18" t="n"/>
+      <c r="G219" s="18" t="n"/>
+      <c r="H219" s="17" t="n"/>
+    </row>
+    <row r="220" ht="19" customHeight="1">
+      <c r="A220" s="16" t="n"/>
+      <c r="B220" s="17" t="n"/>
+      <c r="C220" s="17" t="n"/>
+      <c r="D220" s="16" t="n"/>
+      <c r="E220" s="16" t="n"/>
+      <c r="F220" s="18" t="n"/>
+      <c r="G220" s="18" t="n"/>
+      <c r="H220" s="17" t="n"/>
+    </row>
+    <row r="221" ht="19" customHeight="1">
+      <c r="A221" s="16" t="n"/>
+      <c r="B221" s="17" t="n"/>
+      <c r="C221" s="17" t="n"/>
+      <c r="D221" s="16" t="n"/>
+      <c r="E221" s="16" t="n"/>
+      <c r="F221" s="18" t="n"/>
+      <c r="G221" s="18" t="n"/>
+      <c r="H221" s="17" t="n"/>
+    </row>
+    <row r="222" ht="19" customHeight="1">
+      <c r="A222" s="16" t="n"/>
+      <c r="B222" s="17" t="n"/>
+      <c r="C222" s="17" t="n"/>
+      <c r="D222" s="16" t="n"/>
+      <c r="E222" s="16" t="n"/>
+      <c r="F222" s="18" t="n"/>
+      <c r="G222" s="18" t="n"/>
+      <c r="H222" s="17" t="n"/>
+    </row>
+    <row r="223" ht="19" customHeight="1">
+      <c r="A223" s="16" t="n"/>
+      <c r="B223" s="17" t="n"/>
+      <c r="C223" s="17" t="n"/>
+      <c r="D223" s="16" t="n"/>
+      <c r="E223" s="16" t="n"/>
+      <c r="F223" s="18" t="n"/>
+      <c r="G223" s="18" t="n"/>
+      <c r="H223" s="17" t="n"/>
+    </row>
+    <row r="224" ht="19" customHeight="1">
+      <c r="A224" s="16" t="n"/>
+      <c r="B224" s="17" t="n"/>
+      <c r="C224" s="17" t="n"/>
+      <c r="D224" s="16" t="n"/>
+      <c r="E224" s="16" t="n"/>
+      <c r="F224" s="18" t="n"/>
+      <c r="G224" s="18" t="n"/>
+      <c r="H224" s="17" t="n"/>
+    </row>
+    <row r="225" ht="19" customHeight="1">
+      <c r="A225" s="16" t="n"/>
+      <c r="B225" s="17" t="n"/>
+      <c r="C225" s="17" t="n"/>
+      <c r="D225" s="16" t="n"/>
+      <c r="E225" s="16" t="n"/>
+      <c r="F225" s="18" t="n"/>
+      <c r="G225" s="18" t="n"/>
+      <c r="H225" s="17" t="n"/>
+    </row>
+    <row r="226" ht="19" customHeight="1">
+      <c r="A226" s="16" t="n"/>
+      <c r="B226" s="17" t="n"/>
+      <c r="C226" s="17" t="n"/>
+      <c r="D226" s="16" t="n"/>
+      <c r="E226" s="16" t="n"/>
+      <c r="F226" s="18" t="n"/>
+      <c r="G226" s="18" t="n"/>
+      <c r="H226" s="17" t="n"/>
+    </row>
+    <row r="227" ht="19" customHeight="1">
+      <c r="A227" s="16" t="n"/>
+      <c r="B227" s="17" t="n"/>
+      <c r="C227" s="17" t="n"/>
+      <c r="D227" s="16" t="n"/>
+      <c r="E227" s="16" t="n"/>
+      <c r="F227" s="18" t="n"/>
+      <c r="G227" s="18" t="n"/>
+      <c r="H227" s="17" t="n"/>
+    </row>
+    <row r="228" ht="18" customHeight="1">
+      <c r="A228" s="25" t="inlineStr">
+        <is>
+          <t>※工事内容明細には消費税が含まれておりません。</t>
+        </is>
+      </c>
+    </row>
+    <row r="229" ht="22" customHeight="1">
+      <c r="A229" s="26" t="n"/>
+      <c r="B229" s="26" t="n"/>
+      <c r="C229" s="26" t="n"/>
+      <c r="D229" s="26" t="n"/>
+      <c r="E229" s="26" t="n"/>
+      <c r="F229" s="27" t="inlineStr">
+        <is>
+          <t>合　計</t>
+        </is>
+      </c>
+      <c r="G229" s="28" t="n"/>
+      <c r="H229" s="26" t="n"/>
+    </row>
+    <row r="230" ht="22" customHeight="1">
+      <c r="A230" s="24" t="inlineStr">
+        <is>
+          <t>工 事 内 容 明 細</t>
+        </is>
+      </c>
+    </row>
+    <row r="231" ht="22" customHeight="1">
+      <c r="A231" s="15" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="B231" s="15" t="inlineStr">
+        <is>
+          <t>工事品目</t>
+        </is>
+      </c>
+      <c r="C231" s="15" t="inlineStr">
+        <is>
+          <t>仕様</t>
+        </is>
+      </c>
+      <c r="D231" s="15" t="inlineStr">
+        <is>
+          <t>数量</t>
+        </is>
+      </c>
+      <c r="E231" s="15" t="inlineStr">
+        <is>
+          <t>単位</t>
+        </is>
+      </c>
+      <c r="F231" s="15" t="inlineStr">
+        <is>
+          <t>単価</t>
+        </is>
+      </c>
+      <c r="G231" s="15" t="inlineStr">
+        <is>
+          <t>金額</t>
+        </is>
+      </c>
+      <c r="H231" s="15" t="inlineStr">
+        <is>
+          <t>備考</t>
+        </is>
+      </c>
+    </row>
+    <row r="232" ht="19" customHeight="1">
+      <c r="A232" s="16" t="n"/>
+      <c r="B232" s="17" t="n"/>
+      <c r="C232" s="17" t="n"/>
+      <c r="D232" s="16" t="n"/>
+      <c r="E232" s="16" t="n"/>
+      <c r="F232" s="18" t="n"/>
+      <c r="G232" s="18" t="n"/>
+      <c r="H232" s="17" t="n"/>
+    </row>
+    <row r="233" ht="19" customHeight="1">
+      <c r="A233" s="16" t="n"/>
+      <c r="B233" s="17" t="n"/>
+      <c r="C233" s="17" t="n"/>
+      <c r="D233" s="16" t="n"/>
+      <c r="E233" s="16" t="n"/>
+      <c r="F233" s="18" t="n"/>
+      <c r="G233" s="18" t="n"/>
+      <c r="H233" s="17" t="n"/>
+    </row>
+    <row r="234" ht="19" customHeight="1">
+      <c r="A234" s="16" t="n"/>
+      <c r="B234" s="17" t="n"/>
+      <c r="C234" s="17" t="n"/>
+      <c r="D234" s="16" t="n"/>
+      <c r="E234" s="16" t="n"/>
+      <c r="F234" s="18" t="n"/>
+      <c r="G234" s="18" t="n"/>
+      <c r="H234" s="17" t="n"/>
+    </row>
+    <row r="235" ht="19" customHeight="1">
+      <c r="A235" s="16" t="n"/>
+      <c r="B235" s="17" t="n"/>
+      <c r="C235" s="17" t="n"/>
+      <c r="D235" s="16" t="n"/>
+      <c r="E235" s="16" t="n"/>
+      <c r="F235" s="18" t="n"/>
+      <c r="G235" s="18" t="n"/>
+      <c r="H235" s="17" t="n"/>
+    </row>
+    <row r="236" ht="19" customHeight="1">
+      <c r="A236" s="16" t="n"/>
+      <c r="B236" s="17" t="n"/>
+      <c r="C236" s="17" t="n"/>
+      <c r="D236" s="16" t="n"/>
+      <c r="E236" s="16" t="n"/>
+      <c r="F236" s="18" t="n"/>
+      <c r="G236" s="18" t="n"/>
+      <c r="H236" s="17" t="n"/>
+    </row>
+    <row r="237" ht="19" customHeight="1">
+      <c r="A237" s="16" t="n"/>
+      <c r="B237" s="17" t="n"/>
+      <c r="C237" s="17" t="n"/>
+      <c r="D237" s="16" t="n"/>
+      <c r="E237" s="16" t="n"/>
+      <c r="F237" s="18" t="n"/>
+      <c r="G237" s="18" t="n"/>
+      <c r="H237" s="17" t="n"/>
+    </row>
+    <row r="238" ht="19" customHeight="1">
+      <c r="A238" s="16" t="n"/>
+      <c r="B238" s="17" t="n"/>
+      <c r="C238" s="17" t="n"/>
+      <c r="D238" s="16" t="n"/>
+      <c r="E238" s="16" t="n"/>
+      <c r="F238" s="18" t="n"/>
+      <c r="G238" s="18" t="n"/>
+      <c r="H238" s="17" t="n"/>
+    </row>
+    <row r="239" ht="19" customHeight="1">
+      <c r="A239" s="16" t="n"/>
+      <c r="B239" s="17" t="n"/>
+      <c r="C239" s="17" t="n"/>
+      <c r="D239" s="16" t="n"/>
+      <c r="E239" s="16" t="n"/>
+      <c r="F239" s="18" t="n"/>
+      <c r="G239" s="18" t="n"/>
+      <c r="H239" s="17" t="n"/>
+    </row>
+    <row r="240" ht="19" customHeight="1">
+      <c r="A240" s="16" t="n"/>
+      <c r="B240" s="17" t="n"/>
+      <c r="C240" s="17" t="n"/>
+      <c r="D240" s="16" t="n"/>
+      <c r="E240" s="16" t="n"/>
+      <c r="F240" s="18" t="n"/>
+      <c r="G240" s="18" t="n"/>
+      <c r="H240" s="17" t="n"/>
+    </row>
+    <row r="241" ht="19" customHeight="1">
+      <c r="A241" s="16" t="n"/>
+      <c r="B241" s="17" t="n"/>
+      <c r="C241" s="17" t="n"/>
+      <c r="D241" s="16" t="n"/>
+      <c r="E241" s="16" t="n"/>
+      <c r="F241" s="18" t="n"/>
+      <c r="G241" s="18" t="n"/>
+      <c r="H241" s="17" t="n"/>
+    </row>
+    <row r="242" ht="19" customHeight="1">
+      <c r="A242" s="16" t="n"/>
+      <c r="B242" s="17" t="n"/>
+      <c r="C242" s="17" t="n"/>
+      <c r="D242" s="16" t="n"/>
+      <c r="E242" s="16" t="n"/>
+      <c r="F242" s="18" t="n"/>
+      <c r="G242" s="18" t="n"/>
+      <c r="H242" s="17" t="n"/>
+    </row>
+    <row r="243" ht="19" customHeight="1">
+      <c r="A243" s="16" t="n"/>
+      <c r="B243" s="17" t="n"/>
+      <c r="C243" s="17" t="n"/>
+      <c r="D243" s="16" t="n"/>
+      <c r="E243" s="16" t="n"/>
+      <c r="F243" s="18" t="n"/>
+      <c r="G243" s="18" t="n"/>
+      <c r="H243" s="17" t="n"/>
+    </row>
+    <row r="244" ht="19" customHeight="1">
+      <c r="A244" s="16" t="n"/>
+      <c r="B244" s="17" t="n"/>
+      <c r="C244" s="17" t="n"/>
+      <c r="D244" s="16" t="n"/>
+      <c r="E244" s="16" t="n"/>
+      <c r="F244" s="18" t="n"/>
+      <c r="G244" s="18" t="n"/>
+      <c r="H244" s="17" t="n"/>
+    </row>
+    <row r="245" ht="19" customHeight="1">
+      <c r="A245" s="16" t="n"/>
+      <c r="B245" s="17" t="n"/>
+      <c r="C245" s="17" t="n"/>
+      <c r="D245" s="16" t="n"/>
+      <c r="E245" s="16" t="n"/>
+      <c r="F245" s="18" t="n"/>
+      <c r="G245" s="18" t="n"/>
+      <c r="H245" s="17" t="n"/>
+    </row>
+    <row r="246" ht="19" customHeight="1">
+      <c r="A246" s="16" t="n"/>
+      <c r="B246" s="17" t="n"/>
+      <c r="C246" s="17" t="n"/>
+      <c r="D246" s="16" t="n"/>
+      <c r="E246" s="16" t="n"/>
+      <c r="F246" s="18" t="n"/>
+      <c r="G246" s="18" t="n"/>
+      <c r="H246" s="17" t="n"/>
+    </row>
+    <row r="247" ht="19" customHeight="1">
+      <c r="A247" s="16" t="n"/>
+      <c r="B247" s="17" t="n"/>
+      <c r="C247" s="17" t="n"/>
+      <c r="D247" s="16" t="n"/>
+      <c r="E247" s="16" t="n"/>
+      <c r="F247" s="18" t="n"/>
+      <c r="G247" s="18" t="n"/>
+      <c r="H247" s="17" t="n"/>
+    </row>
+    <row r="248" ht="19" customHeight="1">
+      <c r="A248" s="16" t="n"/>
+      <c r="B248" s="17" t="n"/>
+      <c r="C248" s="17" t="n"/>
+      <c r="D248" s="16" t="n"/>
+      <c r="E248" s="16" t="n"/>
+      <c r="F248" s="18" t="n"/>
+      <c r="G248" s="18" t="n"/>
+      <c r="H248" s="17" t="n"/>
+    </row>
+    <row r="249" ht="19" customHeight="1">
+      <c r="A249" s="16" t="n"/>
+      <c r="B249" s="17" t="n"/>
+      <c r="C249" s="17" t="n"/>
+      <c r="D249" s="16" t="n"/>
+      <c r="E249" s="16" t="n"/>
+      <c r="F249" s="18" t="n"/>
+      <c r="G249" s="18" t="n"/>
+      <c r="H249" s="17" t="n"/>
+    </row>
+    <row r="250" ht="19" customHeight="1">
+      <c r="A250" s="16" t="n"/>
+      <c r="B250" s="17" t="n"/>
+      <c r="C250" s="17" t="n"/>
+      <c r="D250" s="16" t="n"/>
+      <c r="E250" s="16" t="n"/>
+      <c r="F250" s="18" t="n"/>
+      <c r="G250" s="18" t="n"/>
+      <c r="H250" s="17" t="n"/>
+    </row>
+    <row r="251" ht="19" customHeight="1">
+      <c r="A251" s="16" t="n"/>
+      <c r="B251" s="17" t="n"/>
+      <c r="C251" s="17" t="n"/>
+      <c r="D251" s="16" t="n"/>
+      <c r="E251" s="16" t="n"/>
+      <c r="F251" s="18" t="n"/>
+      <c r="G251" s="18" t="n"/>
+      <c r="H251" s="17" t="n"/>
+    </row>
+    <row r="252" ht="18" customHeight="1">
+      <c r="A252" s="25" t="inlineStr">
+        <is>
+          <t>※工事内容明細には消費税が含まれておりません。</t>
+        </is>
+      </c>
+    </row>
+    <row r="253" ht="22" customHeight="1">
+      <c r="A253" s="26" t="n"/>
+      <c r="B253" s="26" t="n"/>
+      <c r="C253" s="26" t="n"/>
+      <c r="D253" s="26" t="n"/>
+      <c r="E253" s="26" t="n"/>
+      <c r="F253" s="27" t="inlineStr">
+        <is>
+          <t>合　計</t>
+        </is>
+      </c>
+      <c r="G253" s="28" t="n"/>
+      <c r="H253" s="26" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="32">
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="E175:F175"/>
+  <mergeCells count="47">
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="E26:H26"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="A53:D53"/>
+    <mergeCell ref="E55:F55"/>
+    <mergeCell ref="C13:E14"/>
     <mergeCell ref="A182:H182"/>
-    <mergeCell ref="E16:H16"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="B179:H180"/>
+    <mergeCell ref="A132:E132"/>
+    <mergeCell ref="E25:H25"/>
     <mergeCell ref="G8:H8"/>
-    <mergeCell ref="C12:E12"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="A110:H110"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="A228:E228"/>
+    <mergeCell ref="A13:B14"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="A5:C5"/>
     <mergeCell ref="G7:H7"/>
-    <mergeCell ref="E177:F177"/>
-    <mergeCell ref="A10:B11"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="E173:F173"/>
-    <mergeCell ref="E176:F176"/>
-    <mergeCell ref="E14:H14"/>
-    <mergeCell ref="C10:E11"/>
-    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="A252:E252"/>
+    <mergeCell ref="A108:E108"/>
+    <mergeCell ref="A84:E84"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A158:H158"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="E59:F59"/>
+    <mergeCell ref="A86:H86"/>
+    <mergeCell ref="A204:E204"/>
+    <mergeCell ref="E58:F58"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="E13:H13"/>
-    <mergeCell ref="A20:H20"/>
-    <mergeCell ref="E174:F174"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="E15:H15"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="E28:H28"/>
+    <mergeCell ref="E57:F57"/>
+    <mergeCell ref="A206:H206"/>
+    <mergeCell ref="A62:H62"/>
+    <mergeCell ref="A180:E180"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A156:E156"/>
+    <mergeCell ref="A134:H134"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="A230:H230"/>
+    <mergeCell ref="E56:F56"/>
+    <mergeCell ref="E27:H27"/>
+    <mergeCell ref="A34:H34"/>
   </mergeCells>
-  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.5" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="85"/>
+  <pageMargins left="0.32" right="0.32" top="0.35" bottom="0.35" header="0.18" footer="0.18"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <rowBreaks count="9" manualBreakCount="9">
+    <brk id="32" min="0" max="16383" man="1"/>
+    <brk id="60" min="0" max="16383" man="1"/>
+    <brk id="85" min="0" max="16383" man="1"/>
+    <brk id="109" min="0" max="16383" man="1"/>
+    <brk id="133" min="0" max="16383" man="1"/>
+    <brk id="157" min="0" max="16383" man="1"/>
+    <brk id="181" min="0" max="16383" man="1"/>
+    <brk id="205" min="0" max="16383" man="1"/>
+    <brk id="229" min="0" max="16383" man="1"/>
+  </rowBreaks>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>